<commit_message>
Prepare submission review with 2000-draw bootstrap and revised reporting
</commit_message>
<xml_diff>
--- a/outputs/Stack-and-reuse/Supplementary-Tables/Supplementary-Tables.xlsx
+++ b/outputs/Stack-and-reuse/Supplementary-Tables/Supplementary-Tables.xlsx
@@ -2,28 +2,29 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Contents" sheetId="1" ns1:id="R6faf48ee4f364b35"/>
-    <sheet name="S1" sheetId="2" ns1:id="Rcd735eb6b43c4442"/>
-    <sheet name="S2" sheetId="3" ns1:id="R882e083dbfe14dcf"/>
-    <sheet name="S3" sheetId="4" ns1:id="R28603e94d4b34147"/>
-    <sheet name="S4" sheetId="5" ns1:id="R668eaa974e3847b8"/>
-    <sheet name="S5" sheetId="6" ns1:id="R2464c7afd8814c49"/>
-    <sheet name="S6" sheetId="7" ns1:id="Rccc85357321e47e6"/>
-    <sheet name="S7" sheetId="8" ns1:id="R2f4e0b8dc1664135"/>
-    <sheet name="S8" sheetId="9" ns1:id="R4019d84ede8e4df4"/>
-    <sheet name="S9" sheetId="10" ns1:id="R16576041fed145ad"/>
-    <sheet name="S10" sheetId="11" ns1:id="Rf4abb955d2fb4ff2"/>
-    <sheet name="S11" sheetId="12" ns1:id="Readd855356344af7"/>
-    <sheet name="S12" sheetId="13" ns1:id="Rfbcdc0595a414ca5"/>
-    <sheet name="S13" sheetId="14" ns1:id="R332fe6b4352f4ae7"/>
-    <sheet name="S14" sheetId="15" ns1:id="R688aec16cc6d4268"/>
-    <sheet name="S15" sheetId="16" ns1:id="R393e235bfd4c4d58"/>
-    <sheet name="S16" sheetId="17" ns1:id="R2ac501d5f0404483"/>
-    <sheet name="S17" sheetId="18" ns1:id="Rc82c2ce9784e444a"/>
-    <sheet name="S18" sheetId="19" ns1:id="R8e7840fc83d1460e"/>
-    <sheet name="S19" sheetId="20" ns1:id="R75d9ab5c37614f48"/>
-    <sheet name="S20" sheetId="21" ns1:id="Ra14b4444d04f4586"/>
-    <sheet name="S21" sheetId="22" ns1:id="R65d4599f1e8443b0"/>
+    <sheet name="Contents" sheetId="1" ns1:id="Rab75b308679f4a33"/>
+    <sheet name="S1" sheetId="2" ns1:id="Rf40c8566242e4e07"/>
+    <sheet name="S2" sheetId="3" ns1:id="Rc76692ae990f4a15"/>
+    <sheet name="S3" sheetId="4" ns1:id="Rcaa81fd2f32446ed"/>
+    <sheet name="S4" sheetId="5" ns1:id="R3859053b867b455f"/>
+    <sheet name="S5" sheetId="6" ns1:id="Rb1d02a3701034aa5"/>
+    <sheet name="S6" sheetId="7" ns1:id="Rbed157908ce14110"/>
+    <sheet name="S7" sheetId="8" ns1:id="Rc561f7f573bc4b97"/>
+    <sheet name="S8" sheetId="9" ns1:id="R00e9148d09374cc2"/>
+    <sheet name="S9" sheetId="10" ns1:id="R40ff1988a2504ec6"/>
+    <sheet name="S10" sheetId="11" ns1:id="R5f11d49826ca40d4"/>
+    <sheet name="S11" sheetId="12" ns1:id="R4077b5bd649f4c38"/>
+    <sheet name="S12" sheetId="13" ns1:id="R41174f8cac674343"/>
+    <sheet name="S13" sheetId="14" ns1:id="R21a0262c146d402c"/>
+    <sheet name="S14" sheetId="15" ns1:id="Rfe904dae251a4268"/>
+    <sheet name="S15" sheetId="16" ns1:id="Rec7fe9f259fb4683"/>
+    <sheet name="S16" sheetId="17" ns1:id="Rb9ad0b636f4a42ac"/>
+    <sheet name="S17" sheetId="18" ns1:id="R7d6e75ea737246db"/>
+    <sheet name="S18" sheetId="19" ns1:id="Re46c724494d6433a"/>
+    <sheet name="S19" sheetId="20" ns1:id="R22d79e6faba14693"/>
+    <sheet name="S20" sheetId="21" ns1:id="R5fe92315e1d04983"/>
+    <sheet name="S21" sheetId="22" ns1:id="R2a757c58164d4563"/>
+    <sheet name="S22" sheetId="23" ns1:id="Rba2ad32a51004f51"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Contents'!$B$2:$E$35</definedName>
@@ -69,6 +70,8 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="20">'S20'!$7:$7,'S20'!$B:$C</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="21">'S21'!$B$2:$F$128</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="21">'S21'!$7:$7,'S21'!$B:$B</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="22">'S22'!$B$2:$K$105</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="22">'S22'!$7:$7</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -79,7 +82,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="9">
+  <x:numFmts count="10">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0&quot;%&quot;"/>
@@ -89,6 +92,7 @@
     <x:numFmt numFmtId="206" formatCode="0.0%"/>
     <x:numFmt numFmtId="207" formatCode="0.000"/>
     <x:numFmt numFmtId="208" formatCode="0.00&quot;%&quot;"/>
+    <x:numFmt numFmtId="209" formatCode="0.00"/>
   </x:numFmts>
   <x:fonts count="8">
     <x:font>
@@ -133,7 +137,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -148,6 +152,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF2E6F9E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF3F6F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2E6F9E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -224,7 +243,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="150">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -629,6 +648,94 @@
     <x:xf numFmtId="202" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="209" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -640,7 +747,7 @@
         <x:color rgb="FFD1495B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFBECEF"/>
         </x:patternFill>
       </x:fill>
@@ -651,7 +758,7 @@
         <x:color rgb="FF986416"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4DF"/>
         </x:patternFill>
       </x:fill>
@@ -662,7 +769,7 @@
         <x:color rgb="FF74716C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF6F4EF"/>
         </x:patternFill>
       </x:fill>
@@ -949,6 +1056,25 @@
     <x:tableColumn id="3" name="Status"/>
     <x:tableColumn id="4" name="Robustness verdict"/>
     <x:tableColumn id="5" name="Wording after review"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table22.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="22" name="PRIDE_S22" displayName="PRIDE_S22" ref="B7:K101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="B7:K101"/>
+  <x:tableColumns count="10">
+    <x:tableColumn id="1" name="Comparison"/>
+    <x:tableColumn id="2" name="Population"/>
+    <x:tableColumn id="3" name="Period or comparison"/>
+    <x:tableColumn id="4" name="Estimate"/>
+    <x:tableColumn id="5" name="Lower bound"/>
+    <x:tableColumn id="6" name="Upper bound"/>
+    <x:tableColumn id="7" name="Meaning of bounds"/>
+    <x:tableColumn id="8" name="Unit"/>
+    <x:tableColumn id="9" name="Definition or qualification"/>
+    <x:tableColumn id="10" name="Source"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1351,7 +1477,7 @@
     <row r="4" ht="23" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="9" t="str">
-        <v>Supplementary tables S1–S21</v>
+        <v>Supplementary tables S1–S22</v>
       </c>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
@@ -1754,12 +1880,20 @@
       </c>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" ht="23" customHeight="1">
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
+      <c r="B32" s="16" t="str">
+        <v>S22</v>
+      </c>
+      <c r="C32" s="26" t="str">
+        <v>Supporting numerical comparisons</v>
+      </c>
+      <c r="D32" s="12" t="str">
+        <v>Supporting comparisons</v>
+      </c>
+      <c r="E32" s="27" t="n">
+        <v>94</v>
+      </c>
       <c r="F32" s="3"/>
     </row>
     <row r="33" ht="23" customHeight="1">
@@ -1841,27 +1975,28 @@
     <mergeCell ref="B35:E35"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B11" location="'S1'!B2" display="S1" tooltip="Open supplementary table S1"/>
-    <hyperlink ref="B12" location="'S2'!B2" display="S2" tooltip="Open supplementary table S2"/>
-    <hyperlink ref="B13" location="'S3'!B2" display="S3" tooltip="Open supplementary table S3"/>
-    <hyperlink ref="B14" location="'S4'!B2" display="S4" tooltip="Open supplementary table S4"/>
-    <hyperlink ref="B15" location="'S5'!B2" display="S5" tooltip="Open supplementary table S5"/>
-    <hyperlink ref="B16" location="'S6'!B2" display="S6" tooltip="Open supplementary table S6"/>
-    <hyperlink ref="B17" location="'S7'!B2" display="S7" tooltip="Open supplementary table S7"/>
-    <hyperlink ref="B18" location="'S8'!B2" display="S8" tooltip="Open supplementary table S8"/>
-    <hyperlink ref="B19" location="'S9'!B2" display="S9" tooltip="Open supplementary table S9"/>
-    <hyperlink ref="B20" location="'S10'!B2" display="S10" tooltip="Open supplementary table S10"/>
-    <hyperlink ref="B21" location="'S11'!B2" display="S11" tooltip="Open supplementary table S11"/>
-    <hyperlink ref="B22" location="'S12'!B2" display="S12" tooltip="Open supplementary table S12"/>
-    <hyperlink ref="B23" location="'S13'!B2" display="S13" tooltip="Open supplementary table S13"/>
-    <hyperlink ref="B24" location="'S14'!B2" display="S14" tooltip="Open supplementary table S14"/>
-    <hyperlink ref="B25" location="'S15'!B2" display="S15" tooltip="Open supplementary table S15"/>
-    <hyperlink ref="B26" location="'S16'!B2" display="S16" tooltip="Open supplementary table S16"/>
-    <hyperlink ref="B27" location="'S17'!B2" display="S17" tooltip="Open supplementary table S17"/>
-    <hyperlink ref="B28" location="'S18'!B2" display="S18" tooltip="Open supplementary table S18"/>
-    <hyperlink ref="B29" location="'S19'!B2" display="S19" tooltip="Open supplementary table S19"/>
-    <hyperlink ref="B30" location="'S20'!B2" display="S20" tooltip="Open supplementary table S20"/>
-    <hyperlink ref="B31" location="'S21'!B2" display="S21" tooltip="Open supplementary table S21"/>
+    <hyperlink ref="B11" location="'S1'!B2"/>
+    <hyperlink ref="B12" location="'S2'!B2"/>
+    <hyperlink ref="B13" location="'S3'!B2"/>
+    <hyperlink ref="B14" location="'S4'!B2"/>
+    <hyperlink ref="B15" location="'S5'!B2"/>
+    <hyperlink ref="B16" location="'S6'!B2"/>
+    <hyperlink ref="B17" location="'S7'!B2"/>
+    <hyperlink ref="B18" location="'S8'!B2"/>
+    <hyperlink ref="B19" location="'S9'!B2"/>
+    <hyperlink ref="B20" location="'S10'!B2"/>
+    <hyperlink ref="B21" location="'S11'!B2"/>
+    <hyperlink ref="B22" location="'S12'!B2"/>
+    <hyperlink ref="B23" location="'S13'!B2"/>
+    <hyperlink ref="B24" location="'S14'!B2"/>
+    <hyperlink ref="B25" location="'S15'!B2"/>
+    <hyperlink ref="B26" location="'S16'!B2"/>
+    <hyperlink ref="B27" location="'S17'!B2"/>
+    <hyperlink ref="B28" location="'S18'!B2"/>
+    <hyperlink ref="B29" location="'S19'!B2"/>
+    <hyperlink ref="B30" location="'S20'!B2"/>
+    <hyperlink ref="B31" location="'S21'!B2"/>
+    <hyperlink ref="B32" location="'S22'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -2699,7 +2834,7 @@
     <mergeCell ref="B45:E45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -2708,7 +2843,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS9&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R951ee0b987804f2c"/>
+    <tablePart ns1:id="R66d6be05a1cd4e79"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3323,7 +3458,7 @@
     <mergeCell ref="B21:E21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -3332,7 +3467,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS10&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R93310e9a8fda4149"/>
+    <tablePart ns1:id="Rb8f37c396c544d80"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4484,7 +4619,7 @@
     <mergeCell ref="B25:G25"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -4493,7 +4628,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS11&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rc6a145580d09437a"/>
+    <tablePart ns1:id="R1c5fed60687147ca"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5045,7 +5180,7 @@
     <mergeCell ref="B25:G25"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -5054,7 +5189,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS12&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R2e185cff09a148d6"/>
+    <tablePart ns1:id="R7ddeb504eec349da"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6398,7 +6533,7 @@
     <mergeCell ref="B33:G33"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -6407,7 +6542,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS13&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rfbc29a51654c47ce"/>
+    <tablePart ns1:id="Re791832050fd4336"/>
   </tableParts>
 </worksheet>
 </file>
@@ -6975,7 +7110,7 @@
     <mergeCell ref="B28:E28"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -6984,7 +7119,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS14&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R5f4e38ca00d9404d"/>
+    <tablePart ns1:id="Rd418388cc8bc42e1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7698,7 +7833,7 @@
     <mergeCell ref="B29:G29"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -7707,7 +7842,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS15&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R30feec6dd44842c1"/>
+    <tablePart ns1:id="Ra4a5b576152c4c34"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8423,7 +8558,7 @@
     <mergeCell ref="B20:G20"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -8432,7 +8567,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS16&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rf4e5108588c742ff"/>
+    <tablePart ns1:id="R599a8289fa3f4e8e"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10034,7 +10169,7 @@
     <mergeCell ref="B35:G35"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -10043,7 +10178,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS17&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R3e1f851e96244e95"/>
+    <tablePart ns1:id="R60520cd5c44a4706"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11011,7 +11146,7 @@
     <mergeCell ref="B30:G30"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -11020,7 +11155,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS18&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rbb122c67b0d34abc"/>
+    <tablePart ns1:id="R2ab19edbda1a458a"/>
   </tableParts>
 </worksheet>
 </file>
@@ -11816,7 +11951,7 @@
     <row r="27" ht="57" customHeight="1">
       <c r="A27" s="3"/>
       <c r="B27" s="12" t="str">
-        <v>All 36,249 PRIDE datasets released 2013–2025. Standard result files = corrected non-generated expanded mzIdentML/mzTab definition. Identifiable results = file names, archive members and table headers (lower bound). Contributor group = hashed PI contact.</v>
+        <v>All 36,249 PRIDE datasets released 2013–2025. Standard result files = corrected non-generated expanded mzIdentML/mzTab definition. Identifiable results = file names, archive members and table headers; rule-based detection with unmeasured sensitivity and false-positive rates. Contributor group = hashed PI contact.</v>
       </c>
       <c r="C27" s="12"/>
       <c r="D27" s="12"/>
@@ -12142,7 +12277,7 @@
     <mergeCell ref="B33:G33"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -12151,7 +12286,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS1&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rbd7f472a9ec94ed9"/>
+    <tablePart ns1:id="Rc6e98756ec9648d6"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17317,7 +17452,7 @@
     <mergeCell ref="B188:G188"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -17326,7 +17461,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS19&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R52443122152f4039"/>
+    <tablePart ns1:id="Rca6caec3cd2f46d1"/>
   </tableParts>
 </worksheet>
 </file>
@@ -17442,7 +17577,7 @@
         <v>0.66</v>
       </c>
       <c r="F8" s="64" t="n">
-        <v>1.17</v>
+        <v>1.19</v>
       </c>
       <c r="G8" s="3"/>
     </row>
@@ -17458,10 +17593,10 @@
         <v>1.71</v>
       </c>
       <c r="E9" s="65" t="n">
-        <v>1.22</v>
+        <v>1.19</v>
       </c>
       <c r="F9" s="65" t="n">
-        <v>2.35</v>
+        <v>2.39</v>
       </c>
       <c r="G9" s="3"/>
     </row>
@@ -17477,10 +17612,10 @@
         <v>4.08</v>
       </c>
       <c r="E10" s="64" t="n">
-        <v>2.29</v>
+        <v>2.38</v>
       </c>
       <c r="F10" s="64" t="n">
-        <v>7.26</v>
+        <v>6.65</v>
       </c>
       <c r="G10" s="3"/>
     </row>
@@ -17496,10 +17631,10 @@
         <v>1.39</v>
       </c>
       <c r="E11" s="65" t="n">
-        <v>1.17</v>
+        <v>1.14</v>
       </c>
       <c r="F11" s="65" t="n">
-        <v>1.71</v>
+        <v>1.7</v>
       </c>
       <c r="G11" s="3"/>
     </row>
@@ -17515,10 +17650,10 @@
         <v>1.28</v>
       </c>
       <c r="E12" s="64" t="n">
-        <v>1.04</v>
+        <v>0.99</v>
       </c>
       <c r="F12" s="64" t="n">
-        <v>1.73</v>
+        <v>1.74</v>
       </c>
       <c r="G12" s="3"/>
     </row>
@@ -17534,10 +17669,10 @@
         <v>1.35</v>
       </c>
       <c r="E13" s="65" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="F13" s="65" t="n">
-        <v>1.49</v>
+        <v>1.52</v>
       </c>
       <c r="G13" s="3"/>
     </row>
@@ -17648,10 +17783,10 @@
         <v>1.04</v>
       </c>
       <c r="E19" s="65" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="F19" s="65" t="n">
-        <v>1.39</v>
+        <v>1.4</v>
       </c>
       <c r="G19" s="3"/>
     </row>
@@ -17667,10 +17802,10 @@
         <v>1.76</v>
       </c>
       <c r="E20" s="64" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="F20" s="64" t="n">
-        <v>2.5</v>
+        <v>2.53</v>
       </c>
       <c r="G20" s="3"/>
     </row>
@@ -17686,10 +17821,10 @@
         <v>8.37</v>
       </c>
       <c r="E21" s="65" t="n">
-        <v>5.97</v>
+        <v>5.73</v>
       </c>
       <c r="F21" s="65" t="n">
-        <v>11.56</v>
+        <v>11.53</v>
       </c>
       <c r="G21" s="3"/>
     </row>
@@ -17705,10 +17840,10 @@
         <v>2</v>
       </c>
       <c r="E22" s="64" t="n">
-        <v>1.6</v>
+        <v>1.63</v>
       </c>
       <c r="F22" s="64" t="n">
-        <v>2.49</v>
+        <v>2.45</v>
       </c>
       <c r="G22" s="3"/>
     </row>
@@ -17724,10 +17859,10 @@
         <v>1.69</v>
       </c>
       <c r="E23" s="65" t="n">
-        <v>1.17</v>
+        <v>1.16</v>
       </c>
       <c r="F23" s="65" t="n">
-        <v>2.69</v>
+        <v>2.75</v>
       </c>
       <c r="G23" s="3"/>
     </row>
@@ -17743,10 +17878,10 @@
         <v>0.74</v>
       </c>
       <c r="E24" s="87" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="F24" s="87" t="n">
-        <v>1.38</v>
+        <v>1.3</v>
       </c>
       <c r="G24" s="3"/>
     </row>
@@ -17813,7 +17948,7 @@
     <row r="31" ht="87" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="12" t="str">
-        <v>Ridge binomial logit GLM with alpha 1e-4 and L1_wt 0; 200 contributor-group bootstrap draws. Predictors: standard files, detected DIA, SDRF, human and Thermo Fisher-only vendor assignment. Adjustment: release year, pooled field/software categories, log10 bytes floored at 1e6, log(1+citations) and missing-citation indicator. See Supplementary Methods for missingness and category reference levels. A4/A5 report crude rate ratios with 1000 group-bootstrap draws. A5 uses release year plus five calendar years among 2013-2020 releases. SDRF direction is not interpretable because files may be added after release.</v>
+        <v>Ridge binomial logit GLM with alpha 1e-4 and L1_wt 0; 2000 contributor-group bootstrap draws. Predictors: standard files, detected DIA, SDRF, human and Thermo Fisher-only vendor assignment. Adjustment: release year, pooled field/software categories, log10 bytes floored at 1e6, log(1+citations) and missing-citation indicator. See Supplementary Methods for missingness and category reference levels. A4/A5 report crude rate ratios with 1000 group-bootstrap draws. A5 uses release year plus five calendar years among 2013-2020 releases. SDRF direction is not interpretable because files may be added after release.</v>
       </c>
       <c r="C31" s="12"/>
       <c r="D31" s="12"/>
@@ -18006,7 +18141,7 @@
     <mergeCell ref="B37:F37"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -18015,7 +18150,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS20&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Ref800e8f925946d3"/>
+    <tablePart ns1:id="Rb6c95b097f144113"/>
   </tableParts>
 </worksheet>
 </file>
@@ -18152,13 +18287,15 @@
         <v>A3</v>
       </c>
       <c r="C10" s="58" t="str">
-        <v>The file classification matches independent references</v>
+        <v>Rule-based file classifications were checked against format references; sensitivity and false-positive rates were not independently measured.</v>
       </c>
       <c r="D10" s="58" t="str">
         <v>V</v>
       </c>
       <c r="E10" s="58"/>
-      <c r="F10" s="58"/>
+      <c r="F10" s="58" t="str">
+        <v>Rule-based file classifications were checked against format references; sensitivity and false-positive rates were not independently measured.</v>
+      </c>
       <c r="G10" s="3"/>
     </row>
     <row r="11" ht="27" customHeight="1">
@@ -18227,16 +18364,16 @@
         <v>B2</v>
       </c>
       <c r="C15" s="59" t="str">
-        <v>Results identifiable only by their header (renamed or re-saved tool output)</v>
+        <v>Table headers identify additional candidate tool outputs. Model-assisted rule review is not independent validation; detected shares are not established lower bounds.</v>
       </c>
       <c r="D15" s="59" t="str">
         <v>S</v>
       </c>
       <c r="E15" s="59" t="str">
-        <v>survives (lower bound)</v>
+        <v>Detection finding retained; independent accuracy validation not performed</v>
       </c>
       <c r="F15" s="59" t="str">
-        <v>382/389 identified tables correctly attributed. Dataset shares under strict signatures: 42.7% and 71.7%. About half of the tables left unidentified are also tool outputs.</v>
+        <v>Table headers identify additional candidate tool outputs. Model-assisted rule review is not independent validation; detected shares are not established lower bounds.</v>
       </c>
       <c r="G15" s="3"/>
     </row>
@@ -18599,14 +18736,14 @@
         <v>G7</v>
       </c>
       <c r="C39" s="59" t="str">
-        <v>Detected DIA, human samples and Thermo Fisher-only vendor assignments associated with qualifying mentions; mentions do not establish reanalysis.</v>
+        <v>DIA and human datasets had higher adjusted odds of qualifying mentions. The Thermo Fisher-only interval included one with 2000 bootstrap draws. Mentions do not establish reanalysis.</v>
       </c>
       <c r="D39" s="59" t="str">
         <v>V</v>
       </c>
       <c r="E39" s="59"/>
       <c r="F39" s="59" t="str">
-        <v>Detected DIA, human samples and Thermo Fisher-only vendor assignments associated with qualifying mentions; mentions do not establish reanalysis.</v>
+        <v>DIA and human datasets had higher adjusted odds of qualifying mentions. The Thermo Fisher-only interval included one with 2000 bootstrap draws. Mentions do not establish reanalysis.</v>
       </c>
       <c r="G39" s="3"/>
     </row>
@@ -19826,7 +19963,7 @@
     <row r="121" ht="42" customHeight="1">
       <c r="A121" s="3"/>
       <c r="B121" s="12" t="str">
-        <v>Status: V verified; W weakened; S single analysis, not yet attacked; X dropped. attack_verdict and corrected_wording come from the robustness attacks and override status where present. Full numbers, denominators and caveats in Findings-ledger.md.</v>
+        <v>Historical review ledger: V verified in the original review; W weakened; S single analysis; X dropped. These labels are not independent validation. Corrected wording includes later reporting qualifications and supersedes historical claims. The 107 rows are not 107 freshly rerun tests. Source: Findings-ledger.md.</v>
       </c>
       <c r="C121" s="12"/>
       <c r="D121" s="12"/>
@@ -20030,7 +20167,7 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -20039,7 +20176,2955 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS21&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Re6a747c84e6048eb"/>
+    <tablePart ns1:id="R632cee017eb349f8"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF2E6F9E"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="3" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="43" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="49" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="32" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="25" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="25" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="66" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="56" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="121"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
+      <c r="D1" s="121"/>
+      <c r="E1" s="121"/>
+      <c r="F1" s="121"/>
+      <c r="G1" s="121"/>
+      <c r="H1" s="121"/>
+      <c r="I1" s="121"/>
+      <c r="J1" s="121"/>
+      <c r="K1" s="121"/>
+      <c r="L1" s="121"/>
+    </row>
+    <row r="2" ht="25" customHeight="1">
+      <c r="A2" s="121"/>
+      <c r="B2" s="123" t="str">
+        <v>SUPPLEMENTARY TABLE S22</v>
+      </c>
+      <c r="C2" s="123"/>
+      <c r="D2" s="123"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="121"/>
+      <c r="I2" s="121"/>
+      <c r="J2" s="121"/>
+      <c r="K2" s="121"/>
+      <c r="L2" s="121"/>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="121"/>
+      <c r="B3" s="125" t="str">
+        <v>Supporting numerical comparisons</v>
+      </c>
+      <c r="C3" s="125"/>
+      <c r="D3" s="125"/>
+      <c r="E3" s="121"/>
+      <c r="F3" s="121"/>
+      <c r="G3" s="121"/>
+      <c r="H3" s="121"/>
+      <c r="I3" s="121"/>
+      <c r="J3" s="121"/>
+      <c r="K3" s="121"/>
+      <c r="L3" s="121"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="121"/>
+      <c r="B4" s="127" t="str">
+        <v>Supporting comparisons at manuscript reporting precision. Population, period and units accompany every estimate.</v>
+      </c>
+      <c r="C4" s="127"/>
+      <c r="D4" s="127"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="121"/>
+      <c r="G4" s="121"/>
+      <c r="H4" s="121"/>
+      <c r="I4" s="121"/>
+      <c r="J4" s="121"/>
+      <c r="K4" s="121"/>
+      <c r="L4" s="121"/>
+    </row>
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="121"/>
+      <c r="B5" s="128"/>
+      <c r="C5" s="128"/>
+      <c r="D5" s="128"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="121"/>
+      <c r="I5" s="121"/>
+      <c r="J5" s="121"/>
+      <c r="K5" s="121"/>
+      <c r="L5" s="121"/>
+    </row>
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="121"/>
+      <c r="B6" s="122" t="str">
+        <v>Contents</v>
+      </c>
+      <c r="C6" s="121"/>
+      <c r="D6" s="121"/>
+      <c r="E6" s="121"/>
+      <c r="F6" s="121"/>
+      <c r="G6" s="121"/>
+      <c r="H6" s="121"/>
+      <c r="I6" s="121"/>
+      <c r="J6" s="121"/>
+      <c r="K6" s="121"/>
+      <c r="L6" s="121"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="121"/>
+      <c r="B7" s="132" t="str">
+        <v>Comparison</v>
+      </c>
+      <c r="C7" s="132" t="str">
+        <v>Population</v>
+      </c>
+      <c r="D7" s="132" t="str">
+        <v>Period or comparison</v>
+      </c>
+      <c r="E7" s="132" t="str">
+        <v>Estimate</v>
+      </c>
+      <c r="F7" s="132" t="str">
+        <v>Lower bound</v>
+      </c>
+      <c r="G7" s="132" t="str">
+        <v>Upper bound</v>
+      </c>
+      <c r="H7" s="132" t="str">
+        <v>Meaning of bounds</v>
+      </c>
+      <c r="I7" s="132" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="J7" s="132" t="str">
+        <v>Definition or qualification</v>
+      </c>
+      <c r="K7" s="132" t="str">
+        <v>Source</v>
+      </c>
+      <c r="L7" s="121"/>
+    </row>
+    <row r="8" ht="43" customHeight="1">
+      <c r="A8" s="121"/>
+      <c r="B8" s="134" t="str">
+        <v>Distinct journals</v>
+      </c>
+      <c r="C8" s="134" t="str">
+        <v>Linked papers with known journal</v>
+      </c>
+      <c r="D8" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E8" s="138" t="n">
+        <v>78</v>
+      </c>
+      <c r="F8" s="142"/>
+      <c r="G8" s="142"/>
+      <c r="H8" s="143" t="str"/>
+      <c r="I8" s="134" t="str">
+        <v>journals</v>
+      </c>
+      <c r="J8" s="134" t="str"/>
+      <c r="K8" s="134" t="str">
+        <v>Table S18</v>
+      </c>
+      <c r="L8" s="121"/>
+    </row>
+    <row r="9" ht="43" customHeight="1">
+      <c r="A9" s="121"/>
+      <c r="B9" s="135" t="str">
+        <v>Distinct journals</v>
+      </c>
+      <c r="C9" s="135" t="str">
+        <v>Linked papers with known journal</v>
+      </c>
+      <c r="D9" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E9" s="139" t="n">
+        <v>627</v>
+      </c>
+      <c r="F9" s="144"/>
+      <c r="G9" s="144"/>
+      <c r="H9" s="145" t="str"/>
+      <c r="I9" s="135" t="str">
+        <v>journals</v>
+      </c>
+      <c r="J9" s="135" t="str"/>
+      <c r="K9" s="135" t="str">
+        <v>Table S18</v>
+      </c>
+      <c r="L9" s="121"/>
+    </row>
+    <row r="10" ht="43" customHeight="1">
+      <c r="A10" s="121"/>
+      <c r="B10" s="134" t="str">
+        <v>Rarefied instrument richness</v>
+      </c>
+      <c r="C10" s="134" t="str">
+        <v>Equal-sized samples of 1,500 datasets</v>
+      </c>
+      <c r="D10" s="134" t="str">
+        <v>2013–2015</v>
+      </c>
+      <c r="E10" s="138" t="n">
+        <v>66</v>
+      </c>
+      <c r="F10" s="142"/>
+      <c r="G10" s="142"/>
+      <c r="H10" s="143" t="str"/>
+      <c r="I10" s="134" t="str">
+        <v>models</v>
+      </c>
+      <c r="J10" s="134" t="str">
+        <v>Richness did not increase despite more even model representation.</v>
+      </c>
+      <c r="K10" s="134" t="str">
+        <v>Table S3; Fig. 1b</v>
+      </c>
+      <c r="L10" s="121"/>
+    </row>
+    <row r="11" ht="43" customHeight="1">
+      <c r="A11" s="121"/>
+      <c r="B11" s="135" t="str">
+        <v>Rarefied instrument richness</v>
+      </c>
+      <c r="C11" s="135" t="str">
+        <v>Equal-sized samples of 1,500 datasets</v>
+      </c>
+      <c r="D11" s="135" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E11" s="139" t="n">
+        <v>62</v>
+      </c>
+      <c r="F11" s="144"/>
+      <c r="G11" s="144"/>
+      <c r="H11" s="145" t="str"/>
+      <c r="I11" s="135" t="str">
+        <v>models</v>
+      </c>
+      <c r="J11" s="135" t="str">
+        <v>Richness did not increase despite more even model representation.</v>
+      </c>
+      <c r="K11" s="135" t="str">
+        <v>Table S3; Fig. 1b</v>
+      </c>
+      <c r="L11" s="121"/>
+    </row>
+    <row r="12" ht="57" customHeight="1">
+      <c r="A12" s="121"/>
+      <c r="B12" s="134" t="str">
+        <v>Diversity comparisons</v>
+      </c>
+      <c r="C12" s="134" t="str">
+        <v>Contributor groups, journals, instrument models and species</v>
+      </c>
+      <c r="D12" s="134" t="str">
+        <v>2023–2025 versus 2013–2015</v>
+      </c>
+      <c r="E12" s="136"/>
+      <c r="F12" s="142"/>
+      <c r="G12" s="142"/>
+      <c r="H12" s="143" t="str"/>
+      <c r="I12" s="134" t="str"/>
+      <c r="J12" s="134" t="str">
+        <v>Direction agreed at orders 1 and 2. At order 2, tools, research subfields, countries and instrument vendors showed no detectable change.</v>
+      </c>
+      <c r="K12" s="134" t="str">
+        <v>Table S3</v>
+      </c>
+      <c r="L12" s="121"/>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="121"/>
+      <c r="B13" s="135" t="str">
+        <v>Timing of effective-number increases</v>
+      </c>
+      <c r="C13" s="135" t="str">
+        <v>Instrument models, journals and tools</v>
+      </c>
+      <c r="D13" s="135" t="str">
+        <v>2013–2025</v>
+      </c>
+      <c r="E13" s="137"/>
+      <c r="F13" s="144"/>
+      <c r="G13" s="144"/>
+      <c r="H13" s="145" t="str"/>
+      <c r="I13" s="135" t="str"/>
+      <c r="J13" s="135" t="str">
+        <v>Instrument models mainly from 2020; journals until 2022; tools only in 2024 and 2025.</v>
+      </c>
+      <c r="K13" s="135" t="str">
+        <v>Table S2; Fig. 1a</v>
+      </c>
+      <c r="L13" s="121"/>
+    </row>
+    <row r="14" ht="43" customHeight="1">
+      <c r="A14" s="121"/>
+      <c r="B14" s="134" t="str">
+        <v>Human samples named</v>
+      </c>
+      <c r="C14" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D14" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E14" s="138" t="n">
+        <v>41</v>
+      </c>
+      <c r="F14" s="142"/>
+      <c r="G14" s="142"/>
+      <c r="H14" s="143" t="str"/>
+      <c r="I14" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J14" s="134" t="str"/>
+      <c r="K14" s="134" t="str">
+        <v>Supplementary Fig. 9; Gallery/data/29-species.csv</v>
+      </c>
+      <c r="L14" s="121"/>
+    </row>
+    <row r="15" ht="43" customHeight="1">
+      <c r="A15" s="121"/>
+      <c r="B15" s="135" t="str">
+        <v>Human samples named</v>
+      </c>
+      <c r="C15" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D15" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E15" s="139" t="n">
+        <v>52</v>
+      </c>
+      <c r="F15" s="144"/>
+      <c r="G15" s="144"/>
+      <c r="H15" s="145" t="str"/>
+      <c r="I15" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J15" s="135" t="str"/>
+      <c r="K15" s="135" t="str">
+        <v>Supplementary Fig. 9; Gallery/data/29-species.csv</v>
+      </c>
+      <c r="L15" s="121"/>
+    </row>
+    <row r="16" ht="43" customHeight="1">
+      <c r="A16" s="121"/>
+      <c r="B16" s="134" t="str">
+        <v>Mouse samples named</v>
+      </c>
+      <c r="C16" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D16" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E16" s="138" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" s="142"/>
+      <c r="G16" s="142"/>
+      <c r="H16" s="143" t="str"/>
+      <c r="I16" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J16" s="134" t="str"/>
+      <c r="K16" s="134" t="str">
+        <v>Supplementary Fig. 9; Gallery/data/29-species.csv</v>
+      </c>
+      <c r="L16" s="121"/>
+    </row>
+    <row r="17" ht="43" customHeight="1">
+      <c r="A17" s="121"/>
+      <c r="B17" s="135" t="str">
+        <v>Mouse samples named</v>
+      </c>
+      <c r="C17" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D17" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E17" s="139" t="n">
+        <v>19</v>
+      </c>
+      <c r="F17" s="144"/>
+      <c r="G17" s="144"/>
+      <c r="H17" s="145" t="str"/>
+      <c r="I17" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J17" s="135" t="str"/>
+      <c r="K17" s="135" t="str">
+        <v>Supplementary Fig. 9; Gallery/data/29-species.csv</v>
+      </c>
+      <c r="L17" s="121"/>
+    </row>
+    <row r="18" ht="43" customHeight="1">
+      <c r="A18" s="121"/>
+      <c r="B18" s="134" t="str">
+        <v>Neither human nor mouse named</v>
+      </c>
+      <c r="C18" s="134" t="str">
+        <v>354 contributor groups present in both periods</v>
+      </c>
+      <c r="D18" s="134" t="str">
+        <v>2013–2016</v>
+      </c>
+      <c r="E18" s="138" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" s="142"/>
+      <c r="G18" s="142"/>
+      <c r="H18" s="143" t="str"/>
+      <c r="I18" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J18" s="134" t="str"/>
+      <c r="K18" s="134" t="str">
+        <v>Findings-ledger.md; Supplementary Fig. 9</v>
+      </c>
+      <c r="L18" s="121"/>
+    </row>
+    <row r="19" ht="43" customHeight="1">
+      <c r="A19" s="121"/>
+      <c r="B19" s="135" t="str">
+        <v>Neither human nor mouse named</v>
+      </c>
+      <c r="C19" s="135" t="str">
+        <v>354 contributor groups present in both periods</v>
+      </c>
+      <c r="D19" s="135" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E19" s="139" t="n">
+        <v>32</v>
+      </c>
+      <c r="F19" s="144"/>
+      <c r="G19" s="144"/>
+      <c r="H19" s="145" t="str"/>
+      <c r="I19" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J19" s="135" t="str"/>
+      <c r="K19" s="135" t="str">
+        <v>Findings-ledger.md; Supplementary Fig. 9</v>
+      </c>
+      <c r="L19" s="121"/>
+    </row>
+    <row r="20" ht="43" customHeight="1">
+      <c r="A20" s="121"/>
+      <c r="B20" s="134" t="str">
+        <v>First-time contributor share</v>
+      </c>
+      <c r="C20" s="134" t="str">
+        <v>Groups with no earlier PRIDE release since 2013</v>
+      </c>
+      <c r="D20" s="134" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E20" s="138" t="n">
+        <v>44</v>
+      </c>
+      <c r="F20" s="142"/>
+      <c r="G20" s="142"/>
+      <c r="H20" s="143" t="str"/>
+      <c r="I20" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J20" s="134" t="str"/>
+      <c r="K20" s="134" t="str">
+        <v>Table S1; Fig. 1c,d</v>
+      </c>
+      <c r="L20" s="121"/>
+    </row>
+    <row r="21" ht="43" customHeight="1">
+      <c r="A21" s="121"/>
+      <c r="B21" s="135" t="str">
+        <v>Growth in country-resolved deposits</v>
+      </c>
+      <c r="C21" s="135" t="str">
+        <v>Datasets from groups with resolved country</v>
+      </c>
+      <c r="D21" s="135" t="str">
+        <v>2023–2025 versus 2016–2018</v>
+      </c>
+      <c r="E21" s="140" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F21" s="144"/>
+      <c r="G21" s="144"/>
+      <c r="H21" s="145" t="str"/>
+      <c r="I21" s="135" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J21" s="135" t="str"/>
+      <c r="K21" s="135" t="str">
+        <v>Table S6; Fig. 1e–g</v>
+      </c>
+      <c r="L21" s="121"/>
+    </row>
+    <row r="22" ht="43" customHeight="1">
+      <c r="A22" s="121"/>
+      <c r="B22" s="134" t="str">
+        <v>Growth in deposits from China</v>
+      </c>
+      <c r="C22" s="134" t="str">
+        <v>Datasets from groups assigned to China</v>
+      </c>
+      <c r="D22" s="134" t="str">
+        <v>2023–2025 versus 2016–2018</v>
+      </c>
+      <c r="E22" s="141" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F22" s="142"/>
+      <c r="G22" s="142"/>
+      <c r="H22" s="143" t="str"/>
+      <c r="I22" s="134" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J22" s="134" t="str">
+        <v>See S6 for the bootstrap bounds at source precision.</v>
+      </c>
+      <c r="K22" s="134" t="str">
+        <v>Table S6; Fig. 1e–g</v>
+      </c>
+      <c r="L22" s="121"/>
+    </row>
+    <row r="23" ht="43" customHeight="1">
+      <c r="A23" s="121"/>
+      <c r="B23" s="135" t="str">
+        <v>Growth in deposits from Germany</v>
+      </c>
+      <c r="C23" s="135" t="str">
+        <v>Datasets from groups assigned to Germany</v>
+      </c>
+      <c r="D23" s="135" t="str">
+        <v>2023–2025 versus 2016–2018</v>
+      </c>
+      <c r="E23" s="140" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F23" s="144"/>
+      <c r="G23" s="144"/>
+      <c r="H23" s="145" t="str"/>
+      <c r="I23" s="135" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J23" s="135" t="str">
+        <v>See S6 for the bootstrap bounds at source precision.</v>
+      </c>
+      <c r="K23" s="135" t="str">
+        <v>Table S6; Fig. 1e–g</v>
+      </c>
+      <c r="L23" s="121"/>
+    </row>
+    <row r="24" ht="43" customHeight="1">
+      <c r="A24" s="121"/>
+      <c r="B24" s="134" t="str">
+        <v>China share of deposits</v>
+      </c>
+      <c r="C24" s="134" t="str">
+        <v>Country-resolved datasets</v>
+      </c>
+      <c r="D24" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E24" s="138" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="142"/>
+      <c r="G24" s="142"/>
+      <c r="H24" s="143" t="str"/>
+      <c r="I24" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J24" s="134" t="str"/>
+      <c r="K24" s="134" t="str">
+        <v>Fig. 1e–g; Table S6</v>
+      </c>
+      <c r="L24" s="121"/>
+    </row>
+    <row r="25" ht="43" customHeight="1">
+      <c r="A25" s="121"/>
+      <c r="B25" s="135" t="str">
+        <v>China share of deposits</v>
+      </c>
+      <c r="C25" s="135" t="str">
+        <v>Country-resolved datasets</v>
+      </c>
+      <c r="D25" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E25" s="139" t="n">
+        <v>15</v>
+      </c>
+      <c r="F25" s="144"/>
+      <c r="G25" s="144"/>
+      <c r="H25" s="145" t="str"/>
+      <c r="I25" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J25" s="135" t="str"/>
+      <c r="K25" s="135" t="str">
+        <v>Fig. 1e–g; Table S6</v>
+      </c>
+      <c r="L25" s="121"/>
+    </row>
+    <row r="26" ht="43" customHeight="1">
+      <c r="A26" s="121"/>
+      <c r="B26" s="134" t="str">
+        <v>Eligible raw-run datasets</v>
+      </c>
+      <c r="C26" s="134" t="str">
+        <v>Datasets with run counts</v>
+      </c>
+      <c r="D26" s="134" t="str">
+        <v>2013–2016</v>
+      </c>
+      <c r="E26" s="138" t="n">
+        <v>2498</v>
+      </c>
+      <c r="F26" s="142"/>
+      <c r="G26" s="142"/>
+      <c r="H26" s="143" t="str"/>
+      <c r="I26" s="134" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J26" s="134" t="str"/>
+      <c r="K26" s="134" t="str">
+        <v>Table S8; Fig. 2a</v>
+      </c>
+      <c r="L26" s="121"/>
+    </row>
+    <row r="27" ht="43" customHeight="1">
+      <c r="A27" s="121"/>
+      <c r="B27" s="135" t="str">
+        <v>Eligible raw-run datasets</v>
+      </c>
+      <c r="C27" s="135" t="str">
+        <v>Datasets with run counts</v>
+      </c>
+      <c r="D27" s="135" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E27" s="139" t="n">
+        <v>15248</v>
+      </c>
+      <c r="F27" s="144"/>
+      <c r="G27" s="144"/>
+      <c r="H27" s="145" t="str"/>
+      <c r="I27" s="135" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J27" s="135" t="str"/>
+      <c r="K27" s="135" t="str">
+        <v>Table S8; Fig. 2a</v>
+      </c>
+      <c r="L27" s="121"/>
+    </row>
+    <row r="28" ht="43" customHeight="1">
+      <c r="A28" s="121"/>
+      <c r="B28" s="134" t="str">
+        <v>Share with at least 100 runs</v>
+      </c>
+      <c r="C28" s="134" t="str">
+        <v>Datasets with run counts</v>
+      </c>
+      <c r="D28" s="134" t="str">
+        <v>2013–2016</v>
+      </c>
+      <c r="E28" s="141" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F28" s="142"/>
+      <c r="G28" s="142"/>
+      <c r="H28" s="143" t="str"/>
+      <c r="I28" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J28" s="134" t="str"/>
+      <c r="K28" s="134" t="str">
+        <v>Table S8; Fig. 2b</v>
+      </c>
+      <c r="L28" s="121"/>
+    </row>
+    <row r="29" ht="43" customHeight="1">
+      <c r="A29" s="121"/>
+      <c r="B29" s="135" t="str">
+        <v>Share with at least 100 runs</v>
+      </c>
+      <c r="C29" s="135" t="str">
+        <v>Datasets with run counts</v>
+      </c>
+      <c r="D29" s="135" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E29" s="139" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="144"/>
+      <c r="G29" s="144"/>
+      <c r="H29" s="145" t="str"/>
+      <c r="I29" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J29" s="135" t="str"/>
+      <c r="K29" s="135" t="str">
+        <v>Table S8; Fig. 2b</v>
+      </c>
+      <c r="L29" s="121"/>
+    </row>
+    <row r="30" ht="43" customHeight="1">
+      <c r="A30" s="121"/>
+      <c r="B30" s="134" t="str">
+        <v>Mean channels per labelled dataset</v>
+      </c>
+      <c r="C30" s="134" t="str">
+        <v>Datasets using isobaric labelling</v>
+      </c>
+      <c r="D30" s="134" t="str">
+        <v>2014</v>
+      </c>
+      <c r="E30" s="138" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="142"/>
+      <c r="G30" s="142"/>
+      <c r="H30" s="143" t="str"/>
+      <c r="I30" s="134" t="str">
+        <v>channels</v>
+      </c>
+      <c r="J30" s="134" t="str">
+        <v>TMTpro replaced iTRAQ; channels distinguish samples measured together in a run.</v>
+      </c>
+      <c r="K30" s="134" t="str">
+        <v>Supplementary Fig. 8; Gallery/data/27-isobaric-plex.csv</v>
+      </c>
+      <c r="L30" s="121"/>
+    </row>
+    <row r="31" ht="43" customHeight="1">
+      <c r="A31" s="121"/>
+      <c r="B31" s="135" t="str">
+        <v>Mean channels per labelled dataset</v>
+      </c>
+      <c r="C31" s="135" t="str">
+        <v>Datasets using isobaric labelling</v>
+      </c>
+      <c r="D31" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E31" s="139" t="n">
+        <v>13</v>
+      </c>
+      <c r="F31" s="144"/>
+      <c r="G31" s="144"/>
+      <c r="H31" s="145" t="str"/>
+      <c r="I31" s="135" t="str">
+        <v>channels</v>
+      </c>
+      <c r="J31" s="135" t="str">
+        <v>TMTpro replaced iTRAQ; channels distinguish samples measured together in a run.</v>
+      </c>
+      <c r="K31" s="135" t="str">
+        <v>Supplementary Fig. 8; Gallery/data/27-isobaric-plex.csv</v>
+      </c>
+      <c r="L31" s="121"/>
+    </row>
+    <row r="32" ht="87" customHeight="1">
+      <c r="A32" s="121"/>
+      <c r="B32" s="134" t="str">
+        <v>Run-count sensitivity analyses</v>
+      </c>
+      <c r="C32" s="134" t="str">
+        <v>Alternative units, counts, composition and strata</v>
+      </c>
+      <c r="D32" s="134" t="str">
+        <v>2013–2016 versus 2023–2025</v>
+      </c>
+      <c r="E32" s="138" t="n">
+        <v>5</v>
+      </c>
+      <c r="F32" s="142"/>
+      <c r="G32" s="142"/>
+      <c r="H32" s="143" t="str"/>
+      <c r="I32" s="134" t="str">
+        <v>analyses</v>
+      </c>
+      <c r="J32" s="134" t="str">
+        <v>Combine datasets from the same paper; exact counts only; collapse fraction-numbered runs; reweight vendor, acquisition mode, labelling, species and submission type to the early composition; stratify by country. The overall median decline persisted.</v>
+      </c>
+      <c r="K32" s="134" t="str">
+        <v>Table S8; Fig. 2c</v>
+      </c>
+      <c r="L32" s="121"/>
+    </row>
+    <row r="33" ht="43" customHeight="1">
+      <c r="A33" s="121"/>
+      <c r="B33" s="135" t="str">
+        <v>Early Bruker subset</v>
+      </c>
+      <c r="C33" s="135" t="str">
+        <v>Datasets naming Bruker instruments in the run-count comparison</v>
+      </c>
+      <c r="D33" s="135" t="str">
+        <v>2013–2016</v>
+      </c>
+      <c r="E33" s="139" t="n">
+        <v>56</v>
+      </c>
+      <c r="F33" s="144"/>
+      <c r="G33" s="144"/>
+      <c r="H33" s="145" t="str"/>
+      <c r="I33" s="135" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J33" s="135" t="str">
+        <v>No detectable decrease for this subset, TMT-labelled datasets or SCIEX-labelled datasets.</v>
+      </c>
+      <c r="K33" s="135" t="str">
+        <v>Table S8</v>
+      </c>
+      <c r="L33" s="121"/>
+    </row>
+    <row r="34" ht="57" customHeight="1">
+      <c r="A34" s="121"/>
+      <c r="B34" s="134" t="str">
+        <v>Within-group versus pooled slope</v>
+      </c>
+      <c r="C34" s="134" t="str">
+        <v>3,456 groups contributing in multiple years; 23,486 datasets</v>
+      </c>
+      <c r="D34" s="134" t="str">
+        <v>Across the study years</v>
+      </c>
+      <c r="E34" s="138" t="n">
+        <v>38</v>
+      </c>
+      <c r="F34" s="142"/>
+      <c r="G34" s="142"/>
+      <c r="H34" s="143" t="str"/>
+      <c r="I34" s="134" t="str">
+        <v>% of pooled slope</v>
+      </c>
+      <c r="J34" s="134" t="str">
+        <v>Slopes of log2 raw-run counts on time, compared on the same datasets. This is not a decomposition of the median decline.</v>
+      </c>
+      <c r="K34" s="134" t="str">
+        <v>Findings-ledger.md; within-group analysis</v>
+      </c>
+      <c r="L34" s="121"/>
+    </row>
+    <row r="35" ht="43" customHeight="1">
+      <c r="A35" s="121"/>
+      <c r="B35" s="135" t="str">
+        <v>Median raw-run size by model</v>
+      </c>
+      <c r="C35" s="135" t="str">
+        <v>Eligible single-model datasets with exact run counts</v>
+      </c>
+      <c r="D35" s="135" t="str">
+        <v>LTQ Orbitrap</v>
+      </c>
+      <c r="E35" s="140" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F35" s="144"/>
+      <c r="G35" s="144"/>
+      <c r="H35" s="145" t="str"/>
+      <c r="I35" s="135" t="str">
+        <v>GB per run</v>
+      </c>
+      <c r="J35" s="135" t="str">
+        <v>Model references: Makarov2006 and Stewart2023. GB = 10^9 bytes.</v>
+      </c>
+      <c r="K35" s="135" t="str">
+        <v>Table S7; Fig. 2d</v>
+      </c>
+      <c r="L35" s="121"/>
+    </row>
+    <row r="36" ht="43" customHeight="1">
+      <c r="A36" s="121"/>
+      <c r="B36" s="134" t="str">
+        <v>Median raw-run size by model</v>
+      </c>
+      <c r="C36" s="134" t="str">
+        <v>Eligible single-model datasets with exact run counts</v>
+      </c>
+      <c r="D36" s="134" t="str">
+        <v>Orbitrap Astral</v>
+      </c>
+      <c r="E36" s="141" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="F36" s="142"/>
+      <c r="G36" s="142"/>
+      <c r="H36" s="143" t="str"/>
+      <c r="I36" s="134" t="str">
+        <v>GB per run</v>
+      </c>
+      <c r="J36" s="134" t="str">
+        <v>Model references: Makarov2006 and Stewart2023. GB = 10^9 bytes.</v>
+      </c>
+      <c r="K36" s="134" t="str">
+        <v>Table S7; Fig. 2d</v>
+      </c>
+      <c r="L36" s="121"/>
+    </row>
+    <row r="37" ht="43" customHeight="1">
+      <c r="A37" s="121"/>
+      <c r="B37" s="135" t="str">
+        <v>Instrument-mix component of run-size change</v>
+      </c>
+      <c r="C37" s="135" t="str">
+        <v>Single identified model and exact raw-run count</v>
+      </c>
+      <c r="D37" s="135" t="str">
+        <v>2023–2025 versus 2014–2016</v>
+      </c>
+      <c r="E37" s="140" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F37" s="144"/>
+      <c r="G37" s="144"/>
+      <c r="H37" s="145" t="str"/>
+      <c r="I37" s="135" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J37" s="135" t="str">
+        <v>Decomposition of change in mean log10 bytes per run. No interval reported for this component in the manuscript.</v>
+      </c>
+      <c r="K37" s="135" t="str">
+        <v>Table S21, H1.4; Fig. 2d</v>
+      </c>
+      <c r="L37" s="121"/>
+    </row>
+    <row r="38" ht="43" customHeight="1">
+      <c r="A38" s="121"/>
+      <c r="B38" s="134" t="str">
+        <v>Within-model component of run-size change</v>
+      </c>
+      <c r="C38" s="134" t="str">
+        <v>Single identified model and exact raw-run count</v>
+      </c>
+      <c r="D38" s="134" t="str">
+        <v>2023–2025 versus 2014–2016</v>
+      </c>
+      <c r="E38" s="141" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F38" s="146" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G38" s="146" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H38" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I38" s="134" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J38" s="134" t="str">
+        <v>Decomposition of change in mean log10 bytes per run.</v>
+      </c>
+      <c r="K38" s="134" t="str">
+        <v>Table S21, H1.4; Fig. 2d</v>
+      </c>
+      <c r="L38" s="121"/>
+    </row>
+    <row r="39" ht="43" customHeight="1">
+      <c r="A39" s="121"/>
+      <c r="B39" s="135" t="str">
+        <v>Bytes held by largest 1% of deposits</v>
+      </c>
+      <c r="C39" s="135" t="str">
+        <v>All listed dataset bytes</v>
+      </c>
+      <c r="D39" s="135" t="str">
+        <v>2013–2025 releases</v>
+      </c>
+      <c r="E39" s="139" t="n">
+        <v>24</v>
+      </c>
+      <c r="F39" s="144"/>
+      <c r="G39" s="144"/>
+      <c r="H39" s="145" t="str"/>
+      <c r="I39" s="135" t="str">
+        <v>% of bytes</v>
+      </c>
+      <c r="J39" s="135" t="str"/>
+      <c r="K39" s="135" t="str">
+        <v>Fig. 2e; Findings-ledger.md</v>
+      </c>
+      <c r="L39" s="121"/>
+    </row>
+    <row r="40" ht="43" customHeight="1">
+      <c r="A40" s="121"/>
+      <c r="B40" s="134" t="str">
+        <v>Raw vendor-format files</v>
+      </c>
+      <c r="C40" s="134" t="str">
+        <v>All listed file bytes</v>
+      </c>
+      <c r="D40" s="134" t="str">
+        <v>2013–2025 releases</v>
+      </c>
+      <c r="E40" s="138" t="n">
+        <v>84</v>
+      </c>
+      <c r="F40" s="142"/>
+      <c r="G40" s="142"/>
+      <c r="H40" s="143" t="str"/>
+      <c r="I40" s="134" t="str">
+        <v>% of bytes</v>
+      </c>
+      <c r="J40" s="134" t="str"/>
+      <c r="K40" s="134" t="str">
+        <v>Fig. 2f; Supplementary Fig. 6</v>
+      </c>
+      <c r="L40" s="121"/>
+    </row>
+    <row r="41" ht="43" customHeight="1">
+      <c r="A41" s="121"/>
+      <c r="B41" s="135" t="str">
+        <v>Thermo Fisher share of instrument assignments</v>
+      </c>
+      <c r="C41" s="135" t="str">
+        <v>One count per identified dataset, split among named models</v>
+      </c>
+      <c r="D41" s="135" t="str">
+        <v>Annual values, 2013–2025</v>
+      </c>
+      <c r="E41" s="137"/>
+      <c r="F41" s="147" t="n">
+        <v>79</v>
+      </c>
+      <c r="G41" s="147" t="n">
+        <v>89</v>
+      </c>
+      <c r="H41" s="145" t="str">
+        <v>Observed annual range</v>
+      </c>
+      <c r="I41" s="135" t="str">
+        <v>% of fractional counts</v>
+      </c>
+      <c r="J41" s="135" t="str">
+        <v>Different from unweighted model shares in S7.</v>
+      </c>
+      <c r="K41" s="135" t="str">
+        <v>Fig. 3a; Gallery/data/14-fleet-history.csv</v>
+      </c>
+      <c r="L41" s="121"/>
+    </row>
+    <row r="42" ht="43" customHeight="1">
+      <c r="A42" s="121"/>
+      <c r="B42" s="134" t="str">
+        <v>Fractional instrument share: LTQ Orbitrap</v>
+      </c>
+      <c r="C42" s="134" t="str">
+        <v>One count per identified dataset, split among named models</v>
+      </c>
+      <c r="D42" s="134" t="str">
+        <v>2013; first year of series</v>
+      </c>
+      <c r="E42" s="138" t="n">
+        <v>40</v>
+      </c>
+      <c r="F42" s="142"/>
+      <c r="G42" s="142"/>
+      <c r="H42" s="143" t="str"/>
+      <c r="I42" s="134" t="str">
+        <v>% of fractional counts</v>
+      </c>
+      <c r="J42" s="134" t="str">
+        <v>The first-year LTQ Orbitrap value is left-censored.</v>
+      </c>
+      <c r="K42" s="134" t="str">
+        <v>Fig. 3a; Supplementary Fig. 2</v>
+      </c>
+      <c r="L42" s="121"/>
+    </row>
+    <row r="43" ht="43" customHeight="1">
+      <c r="A43" s="121"/>
+      <c r="B43" s="135" t="str">
+        <v>Fractional instrument share: Q Exactive</v>
+      </c>
+      <c r="C43" s="135" t="str">
+        <v>One count per identified dataset, split among named models</v>
+      </c>
+      <c r="D43" s="135" t="str">
+        <v>Peak year</v>
+      </c>
+      <c r="E43" s="139" t="n">
+        <v>38</v>
+      </c>
+      <c r="F43" s="144"/>
+      <c r="G43" s="144"/>
+      <c r="H43" s="145" t="str"/>
+      <c r="I43" s="135" t="str">
+        <v>% of fractional counts</v>
+      </c>
+      <c r="J43" s="135" t="str">
+        <v>The first-year LTQ Orbitrap value is left-censored.</v>
+      </c>
+      <c r="K43" s="135" t="str">
+        <v>Fig. 3a; Supplementary Fig. 2</v>
+      </c>
+      <c r="L43" s="121"/>
+    </row>
+    <row r="44" ht="43" customHeight="1">
+      <c r="A44" s="121"/>
+      <c r="B44" s="134" t="str">
+        <v>Fractional instrument share: Q Exactive HF</v>
+      </c>
+      <c r="C44" s="134" t="str">
+        <v>One count per identified dataset, split among named models</v>
+      </c>
+      <c r="D44" s="134" t="str">
+        <v>Peak year</v>
+      </c>
+      <c r="E44" s="138" t="n">
+        <v>19</v>
+      </c>
+      <c r="F44" s="142"/>
+      <c r="G44" s="142"/>
+      <c r="H44" s="143" t="str"/>
+      <c r="I44" s="134" t="str">
+        <v>% of fractional counts</v>
+      </c>
+      <c r="J44" s="134" t="str">
+        <v>The first-year LTQ Orbitrap value is left-censored.</v>
+      </c>
+      <c r="K44" s="134" t="str">
+        <v>Fig. 3a; Supplementary Fig. 2</v>
+      </c>
+      <c r="L44" s="121"/>
+    </row>
+    <row r="45" ht="43" customHeight="1">
+      <c r="A45" s="121"/>
+      <c r="B45" s="135" t="str">
+        <v>timsTOF-labelled datasets</v>
+      </c>
+      <c r="C45" s="135" t="str">
+        <v>Datasets in instrument-share analysis</v>
+      </c>
+      <c r="D45" s="135" t="str">
+        <v>2021</v>
+      </c>
+      <c r="E45" s="140" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F45" s="144"/>
+      <c r="G45" s="144"/>
+      <c r="H45" s="145" t="str"/>
+      <c r="I45" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J45" s="135" t="str">
+        <v>Meier2021 described increasing use in 2021; deposits are not ownership records.</v>
+      </c>
+      <c r="K45" s="135" t="str">
+        <v>Fig. 3a; Gallery/data/14-fleet-history.csv</v>
+      </c>
+      <c r="L45" s="121"/>
+    </row>
+    <row r="46" ht="43" customHeight="1">
+      <c r="A46" s="121"/>
+      <c r="B46" s="134" t="str">
+        <v>timsTOF-labelled datasets</v>
+      </c>
+      <c r="C46" s="134" t="str">
+        <v>Datasets in instrument-share analysis</v>
+      </c>
+      <c r="D46" s="134" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E46" s="138" t="n">
+        <v>13</v>
+      </c>
+      <c r="F46" s="142"/>
+      <c r="G46" s="142"/>
+      <c r="H46" s="143" t="str"/>
+      <c r="I46" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J46" s="134" t="str">
+        <v>Meier2021 described increasing use in 2021; deposits are not ownership records.</v>
+      </c>
+      <c r="K46" s="134" t="str">
+        <v>Fig. 3a; Gallery/data/14-fleet-history.csv</v>
+      </c>
+      <c r="L46" s="121"/>
+    </row>
+    <row r="47" ht="43" customHeight="1">
+      <c r="A47" s="121"/>
+      <c r="B47" s="135" t="str">
+        <v>Software named: MaxQuant</v>
+      </c>
+      <c r="C47" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D47" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E47" s="139" t="n">
+        <v>28</v>
+      </c>
+      <c r="F47" s="144"/>
+      <c r="G47" s="144"/>
+      <c r="H47" s="145" t="str"/>
+      <c r="I47" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J47" s="135" t="str"/>
+      <c r="K47" s="135" t="str">
+        <v>Fig. 3c; Figure-data/Tool-year.csv</v>
+      </c>
+      <c r="L47" s="121"/>
+    </row>
+    <row r="48" ht="43" customHeight="1">
+      <c r="A48" s="121"/>
+      <c r="B48" s="134" t="str">
+        <v>Software named: Proteome Discoverer</v>
+      </c>
+      <c r="C48" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D48" s="134" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E48" s="138" t="n">
+        <v>20</v>
+      </c>
+      <c r="F48" s="142"/>
+      <c r="G48" s="142"/>
+      <c r="H48" s="143" t="str"/>
+      <c r="I48" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J48" s="134" t="str"/>
+      <c r="K48" s="134" t="str">
+        <v>Fig. 3c; Figure-data/Tool-year.csv</v>
+      </c>
+      <c r="L48" s="121"/>
+    </row>
+    <row r="49" ht="43" customHeight="1">
+      <c r="A49" s="121"/>
+      <c r="B49" s="135" t="str">
+        <v>Tool-country pairs with interval excluding 1</v>
+      </c>
+      <c r="C49" s="135" t="str">
+        <v>20 pairs of a tool and its developers’ country</v>
+      </c>
+      <c r="D49" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E49" s="139" t="n">
+        <v>11</v>
+      </c>
+      <c r="F49" s="144"/>
+      <c r="G49" s="144"/>
+      <c r="H49" s="145" t="str"/>
+      <c r="I49" s="135" t="str">
+        <v>pairs</v>
+      </c>
+      <c r="J49" s="135" t="str">
+        <v>95% interval excludes equal naming rates. Developers’ own laboratories included.</v>
+      </c>
+      <c r="K49" s="135" t="str">
+        <v>Fig. 3d; software-geography analysis</v>
+      </c>
+      <c r="L49" s="121"/>
+    </row>
+    <row r="50" ht="43" customHeight="1">
+      <c r="A50" s="121"/>
+      <c r="B50" s="134" t="str">
+        <v>Developer-country naming ratio: Spectronaut</v>
+      </c>
+      <c r="C50" s="134" t="str">
+        <v>Groups in Switzerland versus groups in all countries combined</v>
+      </c>
+      <c r="D50" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E50" s="141" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F50" s="142"/>
+      <c r="G50" s="142"/>
+      <c r="H50" s="143" t="str"/>
+      <c r="I50" s="134" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J50" s="134" t="str">
+        <v>Examples from the reported tool-country comparison. Full intervals remain in Fig. 3d/source data.</v>
+      </c>
+      <c r="K50" s="134" t="str">
+        <v>Fig. 3d; software-geography analysis</v>
+      </c>
+      <c r="L50" s="121"/>
+    </row>
+    <row r="51" ht="43" customHeight="1">
+      <c r="A51" s="121"/>
+      <c r="B51" s="135" t="str">
+        <v>Developer-country naming ratio: Comet</v>
+      </c>
+      <c r="C51" s="135" t="str">
+        <v>Groups in United States versus groups in all countries combined</v>
+      </c>
+      <c r="D51" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E51" s="140" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F51" s="144"/>
+      <c r="G51" s="144"/>
+      <c r="H51" s="145" t="str"/>
+      <c r="I51" s="135" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J51" s="135" t="str">
+        <v>Examples from the reported tool-country comparison. Full intervals remain in Fig. 3d/source data.</v>
+      </c>
+      <c r="K51" s="135" t="str">
+        <v>Fig. 3d; software-geography analysis</v>
+      </c>
+      <c r="L51" s="121"/>
+    </row>
+    <row r="52" ht="43" customHeight="1">
+      <c r="A52" s="121"/>
+      <c r="B52" s="134" t="str">
+        <v>Developer-country naming ratio: MaxQuant</v>
+      </c>
+      <c r="C52" s="134" t="str">
+        <v>Groups in Germany versus groups in all countries combined</v>
+      </c>
+      <c r="D52" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E52" s="141" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F52" s="142"/>
+      <c r="G52" s="142"/>
+      <c r="H52" s="143" t="str"/>
+      <c r="I52" s="134" t="str">
+        <v>fold</v>
+      </c>
+      <c r="J52" s="134" t="str">
+        <v>Examples from the reported tool-country comparison. Full intervals remain in Fig. 3d/source data.</v>
+      </c>
+      <c r="K52" s="134" t="str">
+        <v>Fig. 3d; software-geography analysis</v>
+      </c>
+      <c r="L52" s="121"/>
+    </row>
+    <row r="53" ht="43" customHeight="1">
+      <c r="A53" s="121"/>
+      <c r="B53" s="135" t="str">
+        <v>MaxQuant 1.6-series share by release year</v>
+      </c>
+      <c r="C53" s="135" t="str">
+        <v>MaxQuant datasets released in 2025 with recovered version</v>
+      </c>
+      <c r="D53" s="135" t="str">
+        <v>Release year 2025</v>
+      </c>
+      <c r="E53" s="139" t="n">
+        <v>47</v>
+      </c>
+      <c r="F53" s="144"/>
+      <c r="G53" s="144"/>
+      <c r="H53" s="145" t="str"/>
+      <c r="I53" s="135" t="str">
+        <v>% of versioned datasets</v>
+      </c>
+      <c r="J53" s="135" t="str">
+        <v>First recorded in PRIDE in 2017; a different denominator from submission-year shares.</v>
+      </c>
+      <c r="K53" s="135" t="str">
+        <v>Supplementary Fig. 4; Gallery/data/31-version-streams.csv</v>
+      </c>
+      <c r="L53" s="121"/>
+    </row>
+    <row r="54" ht="43" customHeight="1">
+      <c r="A54" s="121"/>
+      <c r="B54" s="134" t="str">
+        <v>MaxQuant 1.6-series share by submission year</v>
+      </c>
+      <c r="C54" s="134" t="str">
+        <v>361 versioned datasets among 576 submissions naming MaxQuant</v>
+      </c>
+      <c r="D54" s="134" t="str">
+        <v>Submission year 2025</v>
+      </c>
+      <c r="E54" s="138" t="n">
+        <v>40</v>
+      </c>
+      <c r="F54" s="146" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="G54" s="146" t="n">
+        <v>46.58</v>
+      </c>
+      <c r="H54" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I54" s="134" t="str">
+        <v>% of versioned datasets</v>
+      </c>
+      <c r="J54" s="134" t="str">
+        <v>Point estimate rounded as in prose; Table S12 gives 40.17%.</v>
+      </c>
+      <c r="K54" s="134" t="str">
+        <v>Table S12; Supplementary Fig. 4</v>
+      </c>
+      <c r="L54" s="121"/>
+    </row>
+    <row r="55" ht="43" customHeight="1">
+      <c r="A55" s="121"/>
+      <c r="B55" s="135" t="str">
+        <v>DIA-NN 1.8-series share by submission year</v>
+      </c>
+      <c r="C55" s="135" t="str">
+        <v>110 versioned datasets among 331 submissions naming DIA-NN</v>
+      </c>
+      <c r="D55" s="135" t="str">
+        <v>Submission year 2025</v>
+      </c>
+      <c r="E55" s="139" t="n">
+        <v>61</v>
+      </c>
+      <c r="F55" s="147" t="n">
+        <v>48</v>
+      </c>
+      <c r="G55" s="147" t="n">
+        <v>74</v>
+      </c>
+      <c r="H55" s="145" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I55" s="135" t="str">
+        <v>% of versioned datasets</v>
+      </c>
+      <c r="J55" s="135" t="str">
+        <v>Rounded as in prose; Table S12 gives estimates and bounds at source precision.</v>
+      </c>
+      <c r="K55" s="135" t="str">
+        <v>Table S12; Supplementary Fig. 4</v>
+      </c>
+      <c r="L55" s="121"/>
+    </row>
+    <row r="56" ht="43" customHeight="1">
+      <c r="A56" s="121"/>
+      <c r="B56" s="134" t="str">
+        <v>Eligible identification-result datasets</v>
+      </c>
+      <c r="C56" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D56" s="134" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E56" s="138" t="n">
+        <v>6231</v>
+      </c>
+      <c r="F56" s="142"/>
+      <c r="G56" s="142"/>
+      <c r="H56" s="143" t="str"/>
+      <c r="I56" s="134" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J56" s="134" t="str"/>
+      <c r="K56" s="134" t="str">
+        <v>Table S1; Table S13</v>
+      </c>
+      <c r="L56" s="121"/>
+    </row>
+    <row r="57" ht="43" customHeight="1">
+      <c r="A57" s="121"/>
+      <c r="B57" s="135" t="str">
+        <v>Identifiable results: Top-level file names</v>
+      </c>
+      <c r="C57" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D57" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E57" s="139" t="n">
+        <v>59</v>
+      </c>
+      <c r="F57" s="144"/>
+      <c r="G57" s="144"/>
+      <c r="H57" s="145" t="str"/>
+      <c r="I57" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J57" s="135" t="str">
+        <v>Lower-bound detection, not validity or usability.</v>
+      </c>
+      <c r="K57" s="135" t="str">
+        <v>Table S13; Fig. 4c</v>
+      </c>
+      <c r="L57" s="121"/>
+    </row>
+    <row r="58" ht="43" customHeight="1">
+      <c r="A58" s="121"/>
+      <c r="B58" s="134" t="str">
+        <v>Identifiable results: Adding archive contents</v>
+      </c>
+      <c r="C58" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D58" s="134" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E58" s="138" t="n">
+        <v>68</v>
+      </c>
+      <c r="F58" s="142"/>
+      <c r="G58" s="142"/>
+      <c r="H58" s="143" t="str"/>
+      <c r="I58" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J58" s="134" t="str">
+        <v>Lower-bound detection, not validity or usability.</v>
+      </c>
+      <c r="K58" s="134" t="str">
+        <v>Table S13; Fig. 4c</v>
+      </c>
+      <c r="L58" s="121"/>
+    </row>
+    <row r="59" ht="43" customHeight="1">
+      <c r="A59" s="121"/>
+      <c r="B59" s="135" t="str">
+        <v>Identifiable results: Adding table headers</v>
+      </c>
+      <c r="C59" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D59" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E59" s="139" t="n">
+        <v>80</v>
+      </c>
+      <c r="F59" s="144"/>
+      <c r="G59" s="144"/>
+      <c r="H59" s="145" t="str"/>
+      <c r="I59" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J59" s="135" t="str">
+        <v>Lower-bound detection, not validity or usability.</v>
+      </c>
+      <c r="K59" s="135" t="str">
+        <v>Table S13; Fig. 4c</v>
+      </c>
+      <c r="L59" s="121"/>
+    </row>
+    <row r="60" ht="43" customHeight="1">
+      <c r="A60" s="121"/>
+      <c r="B60" s="134" t="str">
+        <v>Identifiable results at all search depths</v>
+      </c>
+      <c r="C60" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D60" s="134" t="str">
+        <v>2015</v>
+      </c>
+      <c r="E60" s="138" t="n">
+        <v>92</v>
+      </c>
+      <c r="F60" s="142"/>
+      <c r="G60" s="142"/>
+      <c r="H60" s="143" t="str"/>
+      <c r="I60" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J60" s="134" t="str">
+        <v>Compared with 80% in 2025.</v>
+      </c>
+      <c r="K60" s="134" t="str">
+        <v>Table S13; Fig. 4d</v>
+      </c>
+      <c r="L60" s="121"/>
+    </row>
+    <row r="61" ht="43" customHeight="1">
+      <c r="A61" s="121"/>
+      <c r="B61" s="135" t="str">
+        <v>Standard-result-file prevalence</v>
+      </c>
+      <c r="C61" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D61" s="135" t="str">
+        <v>Annual values since 2015</v>
+      </c>
+      <c r="E61" s="137"/>
+      <c r="F61" s="147" t="n">
+        <v>16</v>
+      </c>
+      <c r="G61" s="147" t="n">
+        <v>20</v>
+      </c>
+      <c r="H61" s="145" t="str">
+        <v>Observed annual range</v>
+      </c>
+      <c r="I61" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J61" s="135" t="str">
+        <v>Submitter-deposited mzIdentML or mzTab; repository-generated files excluded.</v>
+      </c>
+      <c r="K61" s="135" t="str">
+        <v>Table S13</v>
+      </c>
+      <c r="L61" s="121"/>
+    </row>
+    <row r="62" ht="43" customHeight="1">
+      <c r="A62" s="121"/>
+      <c r="B62" s="134" t="str">
+        <v>Standard result files: DIA-NN</v>
+      </c>
+      <c r="C62" s="134" t="str">
+        <v>Datasets naming a single analysis tool</v>
+      </c>
+      <c r="D62" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E62" s="141" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F62" s="142"/>
+      <c r="G62" s="142"/>
+      <c r="H62" s="143" t="str"/>
+      <c r="I62" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J62" s="134" t="str">
+        <v>Lowest and highest observed tool-specific rates, respectively.</v>
+      </c>
+      <c r="K62" s="134" t="str">
+        <v>Table S9; Fig. 4a</v>
+      </c>
+      <c r="L62" s="121"/>
+    </row>
+    <row r="63" ht="43" customHeight="1">
+      <c r="A63" s="121"/>
+      <c r="B63" s="135" t="str">
+        <v>Standard result files: MS-GF+</v>
+      </c>
+      <c r="C63" s="135" t="str">
+        <v>Datasets naming a single analysis tool</v>
+      </c>
+      <c r="D63" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E63" s="139" t="n">
+        <v>76</v>
+      </c>
+      <c r="F63" s="144"/>
+      <c r="G63" s="144"/>
+      <c r="H63" s="145" t="str"/>
+      <c r="I63" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J63" s="135" t="str">
+        <v>Lowest and highest observed tool-specific rates, respectively.</v>
+      </c>
+      <c r="K63" s="135" t="str">
+        <v>Table S9; Fig. 4a</v>
+      </c>
+      <c r="L63" s="121"/>
+    </row>
+    <row r="64" ht="43" customHeight="1">
+      <c r="A64" s="121"/>
+      <c r="B64" s="134" t="str">
+        <v>Standard files when export is optional</v>
+      </c>
+      <c r="C64" s="134" t="str">
+        <v>Datasets naming tools offering standard output as an option</v>
+      </c>
+      <c r="D64" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E64" s="138" t="n">
+        <v>15</v>
+      </c>
+      <c r="F64" s="148" t="n">
+        <v>14</v>
+      </c>
+      <c r="G64" s="148" t="n">
+        <v>18</v>
+      </c>
+      <c r="H64" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I64" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J64" s="134" t="str"/>
+      <c r="K64" s="134" t="str">
+        <v>Table S10; Fig. 4b</v>
+      </c>
+      <c r="L64" s="121"/>
+    </row>
+    <row r="65" ht="43" customHeight="1">
+      <c r="A65" s="121"/>
+      <c r="B65" s="135" t="str">
+        <v>Default-export group size</v>
+      </c>
+      <c r="C65" s="135" t="str">
+        <v>MS-GF+ and MetaMorpheus only</v>
+      </c>
+      <c r="D65" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E65" s="139" t="n">
+        <v>144</v>
+      </c>
+      <c r="F65" s="144"/>
+      <c r="G65" s="144"/>
+      <c r="H65" s="145" t="str"/>
+      <c r="I65" s="135" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J65" s="135" t="str"/>
+      <c r="K65" s="135" t="str">
+        <v>Table S10; Fig. 4b</v>
+      </c>
+      <c r="L65" s="121"/>
+    </row>
+    <row r="66" ht="43" customHeight="1">
+      <c r="A66" s="121"/>
+      <c r="B66" s="134" t="str">
+        <v>MetaMorpheus deposits with standard files</v>
+      </c>
+      <c r="C66" s="134" t="str">
+        <v>Single-tool MetaMorpheus datasets</v>
+      </c>
+      <c r="D66" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E66" s="138" t="n">
+        <v>23</v>
+      </c>
+      <c r="F66" s="142"/>
+      <c r="G66" s="142"/>
+      <c r="H66" s="143" t="str"/>
+      <c r="I66" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J66" s="134" t="str">
+        <v>The tool writes standard files by default.</v>
+      </c>
+      <c r="K66" s="134" t="str">
+        <v>Table S9; Fig. 4a</v>
+      </c>
+      <c r="L66" s="121"/>
+    </row>
+    <row r="67" ht="43" customHeight="1">
+      <c r="A67" s="121"/>
+      <c r="B67" s="135" t="str">
+        <v>Software-mix component of standard-file change</v>
+      </c>
+      <c r="C67" s="135" t="str">
+        <v>Software families</v>
+      </c>
+      <c r="D67" s="135" t="str">
+        <v>2023–2025 versus 2019–2021</v>
+      </c>
+      <c r="E67" s="139" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F67" s="149" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="G67" s="149" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="H67" s="145" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I67" s="135" t="str">
+        <v>percentage points</v>
+      </c>
+      <c r="J67" s="135" t="str">
+        <v>Mainly growth of DIA-NN and Spectronaut and decline of Mascot.</v>
+      </c>
+      <c r="K67" s="135" t="str">
+        <v>Findings-ledger.md; standards-by-stack analysis</v>
+      </c>
+      <c r="L67" s="121"/>
+    </row>
+    <row r="68" ht="43" customHeight="1">
+      <c r="A68" s="121"/>
+      <c r="B68" s="134" t="str">
+        <v>Within-family component of standard-file change</v>
+      </c>
+      <c r="C68" s="134" t="str">
+        <v>Software families</v>
+      </c>
+      <c r="D68" s="134" t="str">
+        <v>2023–2025 versus 2019–2021</v>
+      </c>
+      <c r="E68" s="141" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F68" s="146" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G68" s="146" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H68" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I68" s="134" t="str">
+        <v>percentage points</v>
+      </c>
+      <c r="J68" s="134" t="str"/>
+      <c r="K68" s="134" t="str">
+        <v>Findings-ledger.md; standards-by-stack analysis</v>
+      </c>
+      <c r="L68" s="121"/>
+    </row>
+    <row r="69" ht="43" customHeight="1">
+      <c r="A69" s="121"/>
+      <c r="B69" s="135" t="str">
+        <v>Standard-file prevalence without detected DIA</v>
+      </c>
+      <c r="C69" s="135" t="str">
+        <v>Datasets with no DIA detected</v>
+      </c>
+      <c r="D69" s="135" t="str">
+        <v>Annual values since 2020</v>
+      </c>
+      <c r="E69" s="137"/>
+      <c r="F69" s="147" t="n">
+        <v>19</v>
+      </c>
+      <c r="G69" s="147" t="n">
+        <v>21</v>
+      </c>
+      <c r="H69" s="145" t="str">
+        <v>Observed annual range</v>
+      </c>
+      <c r="I69" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J69" s="135" t="str"/>
+      <c r="K69" s="135" t="str">
+        <v>Findings-ledger.md; standards-by-stack analysis</v>
+      </c>
+      <c r="L69" s="121"/>
+    </row>
+    <row r="70" ht="43" customHeight="1">
+      <c r="A70" s="121"/>
+      <c r="B70" s="134" t="str">
+        <v>Detected DIA prevalence</v>
+      </c>
+      <c r="C70" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D70" s="134" t="str">
+        <v>2015</v>
+      </c>
+      <c r="E70" s="141" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F70" s="142"/>
+      <c r="G70" s="142"/>
+      <c r="H70" s="143" t="str"/>
+      <c r="I70" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J70" s="134" t="str"/>
+      <c r="K70" s="134" t="str">
+        <v>Table S1; standards-by-stack analysis</v>
+      </c>
+      <c r="L70" s="121"/>
+    </row>
+    <row r="71" ht="43" customHeight="1">
+      <c r="A71" s="121"/>
+      <c r="B71" s="135" t="str">
+        <v>Detected DIA prevalence</v>
+      </c>
+      <c r="C71" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D71" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E71" s="140" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="F71" s="144"/>
+      <c r="G71" s="144"/>
+      <c r="H71" s="145" t="str"/>
+      <c r="I71" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J71" s="135" t="str"/>
+      <c r="K71" s="135" t="str">
+        <v>Table S1; standards-by-stack analysis</v>
+      </c>
+      <c r="L71" s="121"/>
+    </row>
+    <row r="72" ht="43" customHeight="1">
+      <c r="A72" s="121"/>
+      <c r="B72" s="134" t="str">
+        <v>Standard-file prevalence with detected DIA</v>
+      </c>
+      <c r="C72" s="134" t="str">
+        <v>Datasets with DIA detected</v>
+      </c>
+      <c r="D72" s="134" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E72" s="138" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" s="142"/>
+      <c r="G72" s="142"/>
+      <c r="H72" s="143" t="str"/>
+      <c r="I72" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J72" s="134" t="str">
+        <v>Approximately 3%, as reported in prose.</v>
+      </c>
+      <c r="K72" s="134" t="str">
+        <v>Findings-ledger.md; standards-by-stack analysis</v>
+      </c>
+      <c r="L72" s="121"/>
+    </row>
+    <row r="73" ht="57" customHeight="1">
+      <c r="A73" s="121"/>
+      <c r="B73" s="135" t="str">
+        <v>Uncompressed results-archive storage: Scan-level and intermediate search outputs</v>
+      </c>
+      <c r="C73" s="135" t="str">
+        <v>Bytes in uncompressed results archives</v>
+      </c>
+      <c r="D73" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E73" s="139" t="n">
+        <v>66</v>
+      </c>
+      <c r="F73" s="144"/>
+      <c r="G73" s="144"/>
+      <c r="H73" s="145" t="str"/>
+      <c r="I73" s="135" t="str">
+        <v>% of bytes</v>
+      </c>
+      <c r="J73" s="135" t="str"/>
+      <c r="K73" s="135" t="str">
+        <v>Supplementary Fig. 6</v>
+      </c>
+      <c r="L73" s="121"/>
+    </row>
+    <row r="74" ht="43" customHeight="1">
+      <c r="A74" s="121"/>
+      <c r="B74" s="134" t="str">
+        <v>Uncompressed results-archive storage: Final result tables</v>
+      </c>
+      <c r="C74" s="134" t="str">
+        <v>Bytes in uncompressed results archives</v>
+      </c>
+      <c r="D74" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E74" s="141" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F74" s="142"/>
+      <c r="G74" s="142"/>
+      <c r="H74" s="143" t="str"/>
+      <c r="I74" s="134" t="str">
+        <v>% of bytes</v>
+      </c>
+      <c r="J74" s="134" t="str"/>
+      <c r="K74" s="134" t="str">
+        <v>Supplementary Fig. 6</v>
+      </c>
+      <c r="L74" s="121"/>
+    </row>
+    <row r="75" ht="43" customHeight="1">
+      <c r="A75" s="121"/>
+      <c r="B75" s="135" t="str">
+        <v>Spectra in open formats present</v>
+      </c>
+      <c r="C75" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D75" s="135" t="str">
+        <v>2013–2016</v>
+      </c>
+      <c r="E75" s="139" t="n">
+        <v>34</v>
+      </c>
+      <c r="F75" s="144"/>
+      <c r="G75" s="144"/>
+      <c r="H75" s="145" t="str"/>
+      <c r="I75" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J75" s="135" t="str"/>
+      <c r="K75" s="135" t="str">
+        <v>Supplementary Fig. 7; Gallery/data/30-file-formats-periods.csv</v>
+      </c>
+      <c r="L75" s="121"/>
+    </row>
+    <row r="76" ht="43" customHeight="1">
+      <c r="A76" s="121"/>
+      <c r="B76" s="134" t="str">
+        <v>Spectra in open formats present</v>
+      </c>
+      <c r="C76" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D76" s="134" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E76" s="138" t="n">
+        <v>21</v>
+      </c>
+      <c r="F76" s="142"/>
+      <c r="G76" s="142"/>
+      <c r="H76" s="143" t="str"/>
+      <c r="I76" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J76" s="134" t="str"/>
+      <c r="K76" s="134" t="str">
+        <v>Supplementary Fig. 7; Gallery/data/30-file-formats-periods.csv</v>
+      </c>
+      <c r="L76" s="121"/>
+    </row>
+    <row r="77" ht="43" customHeight="1">
+      <c r="A77" s="121"/>
+      <c r="B77" s="135" t="str">
+        <v>Contribution of complete-submission decline</v>
+      </c>
+      <c r="C77" s="135" t="str">
+        <v>Submissions classified as complete require peak lists</v>
+      </c>
+      <c r="D77" s="135" t="str">
+        <v>2013–2016 versus 2023–2025</v>
+      </c>
+      <c r="E77" s="137"/>
+      <c r="F77" s="147" t="n">
+        <v>5</v>
+      </c>
+      <c r="G77" s="147" t="n">
+        <v>10</v>
+      </c>
+      <c r="H77" s="145" t="str">
+        <v>Estimated contribution range</v>
+      </c>
+      <c r="I77" s="135" t="str">
+        <v>percentage points</v>
+      </c>
+      <c r="J77" s="135" t="str">
+        <v>Complete-submission share halved; contribution to the 13 percentage-point open-spectra decline.</v>
+      </c>
+      <c r="K77" s="135" t="str">
+        <v>Supplementary Fig. 7</v>
+      </c>
+      <c r="L77" s="121"/>
+    </row>
+    <row r="78" ht="43" customHeight="1">
+      <c r="A78" s="121"/>
+      <c r="B78" s="134" t="str">
+        <v>SDRF recurrence</v>
+      </c>
+      <c r="C78" s="134" t="str">
+        <v>Next dataset of a group whose previous dataset had SDRF</v>
+      </c>
+      <c r="D78" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E78" s="138" t="n">
+        <v>44</v>
+      </c>
+      <c r="F78" s="142"/>
+      <c r="G78" s="142"/>
+      <c r="H78" s="143" t="str"/>
+      <c r="I78" s="134" t="str">
+        <v>% of next datasets</v>
+      </c>
+      <c r="J78" s="134" t="str">
+        <v>Unadjusted for pairs submitted on the same day or linked to the same paper; includes retrospective additions.</v>
+      </c>
+      <c r="K78" s="134" t="str">
+        <v>Table S14; Fig. 4e</v>
+      </c>
+      <c r="L78" s="121"/>
+    </row>
+    <row r="79" ht="43" customHeight="1">
+      <c r="A79" s="121"/>
+      <c r="B79" s="135" t="str">
+        <v>Expected SDRF recurrence</v>
+      </c>
+      <c r="C79" s="135" t="str">
+        <v>Release-year-matched expectation</v>
+      </c>
+      <c r="D79" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E79" s="140" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F79" s="144"/>
+      <c r="G79" s="144"/>
+      <c r="H79" s="145" t="str"/>
+      <c r="I79" s="135" t="str">
+        <v>% of next datasets</v>
+      </c>
+      <c r="J79" s="135" t="str"/>
+      <c r="K79" s="135" t="str">
+        <v>Table S14; Fig. 4e</v>
+      </c>
+      <c r="L79" s="121"/>
+    </row>
+    <row r="80" ht="43" customHeight="1">
+      <c r="A80" s="121"/>
+      <c r="B80" s="134" t="str">
+        <v>SDRF presence</v>
+      </c>
+      <c r="C80" s="134" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D80" s="134" t="str">
+        <v>2020–2022</v>
+      </c>
+      <c r="E80" s="141" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F80" s="142"/>
+      <c r="G80" s="142"/>
+      <c r="H80" s="143" t="str"/>
+      <c r="I80" s="134" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J80" s="134" t="str"/>
+      <c r="K80" s="134" t="str">
+        <v>Findings-ledger.md; Fig. 4e</v>
+      </c>
+      <c r="L80" s="121"/>
+    </row>
+    <row r="81" ht="43" customHeight="1">
+      <c r="A81" s="121"/>
+      <c r="B81" s="135" t="str">
+        <v>SDRF presence</v>
+      </c>
+      <c r="C81" s="135" t="str">
+        <v>All released datasets</v>
+      </c>
+      <c r="D81" s="135" t="str">
+        <v>2023–2025</v>
+      </c>
+      <c r="E81" s="140" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F81" s="144"/>
+      <c r="G81" s="144"/>
+      <c r="H81" s="145" t="str"/>
+      <c r="I81" s="135" t="str">
+        <v>% of datasets</v>
+      </c>
+      <c r="J81" s="135" t="str"/>
+      <c r="K81" s="135" t="str">
+        <v>Findings-ledger.md; Fig. 4e</v>
+      </c>
+      <c r="L81" s="121"/>
+    </row>
+    <row r="82" ht="43" customHeight="1">
+      <c r="A82" s="121"/>
+      <c r="B82" s="134" t="str">
+        <v>Raw-file measurement-date coverage</v>
+      </c>
+      <c r="C82" s="134" t="str">
+        <v>11,868 dated datasets among 35,364 datasets with raw files</v>
+      </c>
+      <c r="D82" s="134" t="str">
+        <v>2013–2025 releases</v>
+      </c>
+      <c r="E82" s="138" t="n">
+        <v>34</v>
+      </c>
+      <c r="F82" s="142"/>
+      <c r="G82" s="142"/>
+      <c r="H82" s="143" t="str"/>
+      <c r="I82" s="134" t="str">
+        <v>% of raw-file datasets</v>
+      </c>
+      <c r="J82" s="134" t="str"/>
+      <c r="K82" s="134" t="str">
+        <v>Table S15; Fig. 5a</v>
+      </c>
+      <c r="L82" s="121"/>
+    </row>
+    <row r="83" ht="43" customHeight="1">
+      <c r="A83" s="121"/>
+      <c r="B83" s="135" t="str">
+        <v>Database date to public release</v>
+      </c>
+      <c r="C83" s="135" t="str">
+        <v>2,558 datasets with eligible sequence-database date</v>
+      </c>
+      <c r="D83" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E83" s="140" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F83" s="149" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G83" s="149" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="H83" s="145" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I83" s="135" t="str">
+        <v>years</v>
+      </c>
+      <c r="J83" s="135" t="str">
+        <v>Median interval; main dated FASTA represents a dataset.</v>
+      </c>
+      <c r="K83" s="135" t="str">
+        <v>Table S15; Fig. 5a</v>
+      </c>
+      <c r="L83" s="121"/>
+    </row>
+    <row r="84" ht="43" customHeight="1">
+      <c r="A84" s="121"/>
+      <c r="B84" s="134" t="str">
+        <v>Software first appearance to public release</v>
+      </c>
+      <c r="C84" s="134" t="str">
+        <v>10,466 datasets with recovered software-release timing</v>
+      </c>
+      <c r="D84" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E84" s="141" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F84" s="146" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G84" s="146" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H84" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I84" s="134" t="str">
+        <v>years</v>
+      </c>
+      <c r="J84" s="134" t="str">
+        <v>Median is a lower bound measured from first recorded PRIDE appearance.</v>
+      </c>
+      <c r="K84" s="134" t="str">
+        <v>Table S11; Supplementary Fig. 5</v>
+      </c>
+      <c r="L84" s="121"/>
+    </row>
+    <row r="85" ht="43" customHeight="1">
+      <c r="A85" s="121"/>
+      <c r="B85" s="135" t="str">
+        <v>Database date precedes latest measurement</v>
+      </c>
+      <c r="C85" s="135" t="str">
+        <v>1,006 datasets with both relevant dates</v>
+      </c>
+      <c r="D85" s="135" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E85" s="139" t="n">
+        <v>71</v>
+      </c>
+      <c r="F85" s="144"/>
+      <c r="G85" s="144"/>
+      <c r="H85" s="145" t="str"/>
+      <c r="I85" s="135" t="str">
+        <v>% of paired datasets</v>
+      </c>
+      <c r="J85" s="135" t="str"/>
+      <c r="K85" s="135" t="str">
+        <v>Table S15; Fig. 5a</v>
+      </c>
+      <c r="L85" s="121"/>
+    </row>
+    <row r="86" ht="43" customHeight="1">
+      <c r="A86" s="121"/>
+      <c r="B86" s="134" t="str">
+        <v>Software first appearance precedes latest measurement</v>
+      </c>
+      <c r="C86" s="134" t="str">
+        <v>3,986 datasets with both relevant dates</v>
+      </c>
+      <c r="D86" s="134" t="str">
+        <v>Study cohort</v>
+      </c>
+      <c r="E86" s="138" t="n">
+        <v>79</v>
+      </c>
+      <c r="F86" s="142"/>
+      <c r="G86" s="142"/>
+      <c r="H86" s="143" t="str"/>
+      <c r="I86" s="134" t="str">
+        <v>% of paired datasets</v>
+      </c>
+      <c r="J86" s="134" t="str"/>
+      <c r="K86" s="134" t="str">
+        <v>Table S15; Fig. 5a</v>
+      </c>
+      <c r="L86" s="121"/>
+    </row>
+    <row r="87" ht="43" customHeight="1">
+      <c r="A87" s="121"/>
+      <c r="B87" s="135" t="str">
+        <v>Days with clustered public releases</v>
+      </c>
+      <c r="C87" s="135" t="str">
+        <v>At least 50 datasets made public on a day</v>
+      </c>
+      <c r="D87" s="135" t="str">
+        <v>From October 2018 onwards</v>
+      </c>
+      <c r="E87" s="139" t="n">
+        <v>62</v>
+      </c>
+      <c r="F87" s="144"/>
+      <c r="G87" s="144"/>
+      <c r="H87" s="145" t="str"/>
+      <c r="I87" s="135" t="str">
+        <v>days</v>
+      </c>
+      <c r="J87" s="135" t="str"/>
+      <c r="K87" s="135" t="str">
+        <v>Table S16; Supplementary Fig. 13</v>
+      </c>
+      <c r="L87" s="121"/>
+    </row>
+    <row r="88" ht="43" customHeight="1">
+      <c r="A88" s="121"/>
+      <c r="B88" s="134" t="str">
+        <v>Median publication-to-release delay</v>
+      </c>
+      <c r="C88" s="134" t="str">
+        <v>Days with at least 50 public releases</v>
+      </c>
+      <c r="D88" s="134" t="str">
+        <v>From October 2018 onwards</v>
+      </c>
+      <c r="E88" s="138" t="n">
+        <v>95</v>
+      </c>
+      <c r="F88" s="142"/>
+      <c r="G88" s="142"/>
+      <c r="H88" s="143" t="str"/>
+      <c r="I88" s="134" t="str">
+        <v>days</v>
+      </c>
+      <c r="J88" s="134" t="str">
+        <v>Who set the release date is not recorded.</v>
+      </c>
+      <c r="K88" s="134" t="str">
+        <v>Table S16; Supplementary Fig. 13</v>
+      </c>
+      <c r="L88" s="121"/>
+    </row>
+    <row r="89" ht="43" customHeight="1">
+      <c r="A89" s="121"/>
+      <c r="B89" s="135" t="str">
+        <v>Median publication-to-release delay</v>
+      </c>
+      <c r="C89" s="135" t="str">
+        <v>Other days</v>
+      </c>
+      <c r="D89" s="135" t="str">
+        <v>From October 2018 onwards</v>
+      </c>
+      <c r="E89" s="139" t="n">
+        <v>11</v>
+      </c>
+      <c r="F89" s="144"/>
+      <c r="G89" s="144"/>
+      <c r="H89" s="145" t="str"/>
+      <c r="I89" s="135" t="str">
+        <v>days</v>
+      </c>
+      <c r="J89" s="135" t="str">
+        <v>Who set the release date is not recorded.</v>
+      </c>
+      <c r="K89" s="135" t="str">
+        <v>Table S16; Supplementary Fig. 13</v>
+      </c>
+      <c r="L89" s="121"/>
+    </row>
+    <row r="90" ht="43" customHeight="1">
+      <c r="A90" s="121"/>
+      <c r="B90" s="134" t="str">
+        <v>Papers in journals with proteom in title</v>
+      </c>
+      <c r="C90" s="134" t="str">
+        <v>PRIDE-linked papers</v>
+      </c>
+      <c r="D90" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E90" s="138" t="n">
+        <v>142</v>
+      </c>
+      <c r="F90" s="142"/>
+      <c r="G90" s="142"/>
+      <c r="H90" s="143" t="str"/>
+      <c r="I90" s="134" t="str">
+        <v>papers</v>
+      </c>
+      <c r="J90" s="134" t="str"/>
+      <c r="K90" s="134" t="str">
+        <v>Table S17; Fig. 5b,c</v>
+      </c>
+      <c r="L90" s="121"/>
+    </row>
+    <row r="91" ht="43" customHeight="1">
+      <c r="A91" s="121"/>
+      <c r="B91" s="135" t="str">
+        <v>Papers in journals with proteom in title</v>
+      </c>
+      <c r="C91" s="135" t="str">
+        <v>PRIDE-linked papers</v>
+      </c>
+      <c r="D91" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E91" s="139" t="n">
+        <v>259</v>
+      </c>
+      <c r="F91" s="144"/>
+      <c r="G91" s="144"/>
+      <c r="H91" s="145" t="str"/>
+      <c r="I91" s="135" t="str">
+        <v>papers</v>
+      </c>
+      <c r="J91" s="135" t="str"/>
+      <c r="K91" s="135" t="str">
+        <v>Table S17; Fig. 5b,c</v>
+      </c>
+      <c r="L91" s="121"/>
+    </row>
+    <row r="92" ht="43" customHeight="1">
+      <c r="A92" s="121"/>
+      <c r="B92" s="134" t="str">
+        <v>Top-ten journal concentration</v>
+      </c>
+      <c r="C92" s="134" t="str">
+        <v>PRIDE-linked papers</v>
+      </c>
+      <c r="D92" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E92" s="138" t="n">
+        <v>66</v>
+      </c>
+      <c r="F92" s="142"/>
+      <c r="G92" s="142"/>
+      <c r="H92" s="143" t="str"/>
+      <c r="I92" s="134" t="str">
+        <v>% of papers</v>
+      </c>
+      <c r="J92" s="134" t="str"/>
+      <c r="K92" s="134" t="str">
+        <v>Table S18; Fig. 5c</v>
+      </c>
+      <c r="L92" s="121"/>
+    </row>
+    <row r="93" ht="43" customHeight="1">
+      <c r="A93" s="121"/>
+      <c r="B93" s="135" t="str">
+        <v>Top-ten journal concentration</v>
+      </c>
+      <c r="C93" s="135" t="str">
+        <v>PRIDE-linked papers</v>
+      </c>
+      <c r="D93" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E93" s="139" t="n">
+        <v>31</v>
+      </c>
+      <c r="F93" s="144"/>
+      <c r="G93" s="144"/>
+      <c r="H93" s="145" t="str"/>
+      <c r="I93" s="135" t="str">
+        <v>% of papers</v>
+      </c>
+      <c r="J93" s="135" t="str"/>
+      <c r="K93" s="135" t="str">
+        <v>Table S18; Fig. 5c</v>
+      </c>
+      <c r="L93" s="121"/>
+    </row>
+    <row r="94" ht="43" customHeight="1">
+      <c r="A94" s="121"/>
+      <c r="B94" s="134" t="str">
+        <v>Chemistry research-field assignment</v>
+      </c>
+      <c r="C94" s="134" t="str">
+        <v>Linked datasets with research-field assignment</v>
+      </c>
+      <c r="D94" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E94" s="138" t="n">
+        <v>26</v>
+      </c>
+      <c r="F94" s="142"/>
+      <c r="G94" s="142"/>
+      <c r="H94" s="143" t="str"/>
+      <c r="I94" s="134" t="str">
+        <v>% of linked datasets</v>
+      </c>
+      <c r="J94" s="134" t="str">
+        <v>Almost all chemistry assignments were spectroscopy.</v>
+      </c>
+      <c r="K94" s="134" t="str">
+        <v>Supplementary Fig. 12; Gallery/data/36-research-fields-by-year.csv</v>
+      </c>
+      <c r="L94" s="121"/>
+    </row>
+    <row r="95" ht="43" customHeight="1">
+      <c r="A95" s="121"/>
+      <c r="B95" s="135" t="str">
+        <v>Chemistry research-field assignment</v>
+      </c>
+      <c r="C95" s="135" t="str">
+        <v>Linked datasets with research-field assignment</v>
+      </c>
+      <c r="D95" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E95" s="139" t="n">
+        <v>6</v>
+      </c>
+      <c r="F95" s="144"/>
+      <c r="G95" s="144"/>
+      <c r="H95" s="145" t="str"/>
+      <c r="I95" s="135" t="str">
+        <v>% of linked datasets</v>
+      </c>
+      <c r="J95" s="135" t="str">
+        <v>Almost all chemistry assignments were spectroscopy.</v>
+      </c>
+      <c r="K95" s="135" t="str">
+        <v>Supplementary Fig. 12; Gallery/data/36-research-fields-by-year.csv</v>
+      </c>
+      <c r="L95" s="121"/>
+    </row>
+    <row r="96" ht="43" customHeight="1">
+      <c r="A96" s="121"/>
+      <c r="B96" s="134" t="str">
+        <v>Medicine research-field assignment</v>
+      </c>
+      <c r="C96" s="134" t="str">
+        <v>Linked datasets with research-field assignment</v>
+      </c>
+      <c r="D96" s="134" t="str">
+        <v>2013</v>
+      </c>
+      <c r="E96" s="138" t="n">
+        <v>18</v>
+      </c>
+      <c r="F96" s="142"/>
+      <c r="G96" s="142"/>
+      <c r="H96" s="143" t="str"/>
+      <c r="I96" s="134" t="str">
+        <v>% of linked datasets</v>
+      </c>
+      <c r="J96" s="134" t="str"/>
+      <c r="K96" s="134" t="str">
+        <v>Supplementary Fig. 12; Gallery/data/36-research-fields-by-year.csv</v>
+      </c>
+      <c r="L96" s="121"/>
+    </row>
+    <row r="97" ht="43" customHeight="1">
+      <c r="A97" s="121"/>
+      <c r="B97" s="135" t="str">
+        <v>Medicine research-field assignment</v>
+      </c>
+      <c r="C97" s="135" t="str">
+        <v>Linked datasets with research-field assignment</v>
+      </c>
+      <c r="D97" s="135" t="str">
+        <v>2025</v>
+      </c>
+      <c r="E97" s="139" t="n">
+        <v>29</v>
+      </c>
+      <c r="F97" s="144"/>
+      <c r="G97" s="144"/>
+      <c r="H97" s="145" t="str"/>
+      <c r="I97" s="135" t="str">
+        <v>% of linked datasets</v>
+      </c>
+      <c r="J97" s="135" t="str"/>
+      <c r="K97" s="135" t="str">
+        <v>Supplementary Fig. 12; Gallery/data/36-research-fields-by-year.csv</v>
+      </c>
+      <c r="L97" s="121"/>
+    </row>
+    <row r="98" ht="57" customHeight="1">
+      <c r="A98" s="121"/>
+      <c r="B98" s="134" t="str">
+        <v>Qualifying mention analysis population</v>
+      </c>
+      <c r="C98" s="134" t="str">
+        <v>Datasets released in 2013–2022</v>
+      </c>
+      <c r="D98" s="134" t="str">
+        <v>Release calendar year and next three calendar years</v>
+      </c>
+      <c r="E98" s="138" t="n">
+        <v>20684</v>
+      </c>
+      <c r="F98" s="142"/>
+      <c r="G98" s="142"/>
+      <c r="H98" s="143" t="str"/>
+      <c r="I98" s="134" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J98" s="134" t="str">
+        <v>Mentioning paper is not primary reference, names at least 2 contributor groups and no more than 100 datasets. Same-year chronology is unresolved.</v>
+      </c>
+      <c r="K98" s="134" t="str">
+        <v>Table S19; Methods</v>
+      </c>
+      <c r="L98" s="121"/>
+    </row>
+    <row r="99" ht="43" customHeight="1">
+      <c r="A99" s="121"/>
+      <c r="B99" s="135" t="str">
+        <v>Extended-window standard-file rate ratio</v>
+      </c>
+      <c r="C99" s="135" t="str">
+        <v>2013–2020 releases; 11,741 datasets</v>
+      </c>
+      <c r="D99" s="135" t="str">
+        <v>Release calendar year and next five calendar years</v>
+      </c>
+      <c r="E99" s="140" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="F99" s="149" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G99" s="149" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H99" s="145" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I99" s="135" t="str">
+        <v>unadjusted rate ratio</v>
+      </c>
+      <c r="J99" s="135" t="str"/>
+      <c r="K99" s="135" t="str">
+        <v>Table S20; Supplementary Methods</v>
+      </c>
+      <c r="L99" s="121"/>
+    </row>
+    <row r="100" ht="57" customHeight="1">
+      <c r="A100" s="121"/>
+      <c r="B100" s="134" t="str">
+        <v>Restricted-cohort standard-file rate ratio</v>
+      </c>
+      <c r="C100" s="134" t="str">
+        <v>4,399 human datasets; Thermo Fisher only; no DIA detected; MaxQuant or Proteome Discoverer</v>
+      </c>
+      <c r="D100" s="134" t="str">
+        <v>2013–2022 releases; main mention window</v>
+      </c>
+      <c r="E100" s="141" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="F100" s="146" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="G100" s="146" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H100" s="143" t="str">
+        <v>95% interval</v>
+      </c>
+      <c r="I100" s="134" t="str">
+        <v>unadjusted rate ratio</v>
+      </c>
+      <c r="J100" s="134" t="str">
+        <v>These restrictions do not establish raw-file presence or confirm DDA.</v>
+      </c>
+      <c r="K100" s="134" t="str">
+        <v>Table S20; Supplementary Methods</v>
+      </c>
+      <c r="L100" s="121"/>
+    </row>
+    <row r="101" ht="43" customHeight="1">
+      <c r="A101" s="121"/>
+      <c r="B101" s="135" t="str">
+        <v>SDRF datasets released before format existed</v>
+      </c>
+      <c r="C101" s="135" t="str">
+        <v>205 SDRF datasets in the mention-model cohort</v>
+      </c>
+      <c r="D101" s="135" t="str">
+        <v>Release before availability of the SDRF format</v>
+      </c>
+      <c r="E101" s="139" t="n">
+        <v>91</v>
+      </c>
+      <c r="F101" s="144"/>
+      <c r="G101" s="144"/>
+      <c r="H101" s="145" t="str"/>
+      <c r="I101" s="135" t="str">
+        <v>datasets</v>
+      </c>
+      <c r="J101" s="135" t="str">
+        <v>Files added later, often through reanalysis projects; temporal direction of the association is unresolved.</v>
+      </c>
+      <c r="K101" s="135" t="str">
+        <v>Table S20; Findings-ledger.md</v>
+      </c>
+      <c r="L101" s="121"/>
+    </row>
+    <row r="102" ht="25" customHeight="1">
+      <c r="A102" s="121"/>
+      <c r="B102" s="121"/>
+      <c r="C102" s="121"/>
+      <c r="D102" s="121"/>
+      <c r="E102" s="121"/>
+      <c r="F102" s="121"/>
+      <c r="G102" s="121"/>
+      <c r="H102" s="121"/>
+      <c r="I102" s="121"/>
+      <c r="J102" s="121"/>
+      <c r="K102" s="121"/>
+      <c r="L102" s="121"/>
+    </row>
+    <row r="103" ht="25" customHeight="1">
+      <c r="A103" s="121"/>
+      <c r="B103" s="121"/>
+      <c r="C103" s="121"/>
+      <c r="D103" s="121"/>
+      <c r="E103" s="121"/>
+      <c r="F103" s="121"/>
+      <c r="G103" s="121"/>
+      <c r="H103" s="121"/>
+      <c r="I103" s="121"/>
+      <c r="J103" s="121"/>
+      <c r="K103" s="121"/>
+      <c r="L103" s="121"/>
+    </row>
+    <row r="104" ht="25" customHeight="1">
+      <c r="A104" s="121"/>
+      <c r="B104" s="123" t="str">
+        <v>Definition and provenance</v>
+      </c>
+      <c r="C104" s="123"/>
+      <c r="D104" s="123"/>
+      <c r="E104" s="121"/>
+      <c r="F104" s="121"/>
+      <c r="G104" s="121"/>
+      <c r="H104" s="121"/>
+      <c r="I104" s="121"/>
+      <c r="J104" s="121"/>
+      <c r="K104" s="121"/>
+      <c r="L104" s="121"/>
+    </row>
+    <row r="105" ht="70" customHeight="1">
+      <c r="A105" s="121"/>
+      <c r="B105" s="127" t="str">
+        <v>Reported comparisons supporting the Results. Values retain manuscript rounding; source tables retain full precision. Bounds are explicitly labelled as 95% intervals or observed/estimated ranges. Blank bounds mean no interval was reported here, not zero uncertainty. This is a curated reporting table, not a new analysis.</v>
+      </c>
+      <c r="C105" s="127"/>
+      <c r="D105" s="127"/>
+      <c r="E105" s="121"/>
+      <c r="F105" s="121"/>
+      <c r="G105" s="121"/>
+      <c r="H105" s="121"/>
+      <c r="I105" s="121"/>
+      <c r="J105" s="121"/>
+      <c r="K105" s="121"/>
+      <c r="L105" s="121"/>
+    </row>
+    <row r="106" ht="25" customHeight="1">
+      <c r="A106" s="121"/>
+      <c r="B106" s="121"/>
+      <c r="C106" s="121"/>
+      <c r="D106" s="121"/>
+      <c r="E106" s="121"/>
+      <c r="F106" s="121"/>
+      <c r="G106" s="121"/>
+      <c r="H106" s="121"/>
+      <c r="I106" s="121"/>
+      <c r="J106" s="121"/>
+      <c r="K106" s="121"/>
+      <c r="L106" s="121"/>
+    </row>
+    <row r="107" ht="25" customHeight="1">
+      <c r="A107" s="121"/>
+      <c r="B107" s="121"/>
+      <c r="C107" s="121"/>
+      <c r="D107" s="121"/>
+      <c r="E107" s="121"/>
+      <c r="F107" s="121"/>
+      <c r="G107" s="121"/>
+      <c r="H107" s="121"/>
+      <c r="I107" s="121"/>
+      <c r="J107" s="121"/>
+      <c r="K107" s="121"/>
+      <c r="L107" s="121"/>
+    </row>
+    <row r="108" ht="25" customHeight="1">
+      <c r="A108" s="121"/>
+      <c r="B108" s="121"/>
+      <c r="C108" s="121"/>
+      <c r="D108" s="121"/>
+      <c r="E108" s="121"/>
+      <c r="F108" s="121"/>
+      <c r="G108" s="121"/>
+      <c r="H108" s="121"/>
+      <c r="I108" s="121"/>
+      <c r="J108" s="121"/>
+      <c r="K108" s="121"/>
+      <c r="L108" s="121"/>
+    </row>
+    <row r="109" ht="25" customHeight="1">
+      <c r="A109" s="121"/>
+      <c r="B109" s="121"/>
+      <c r="C109" s="121"/>
+      <c r="D109" s="121"/>
+      <c r="E109" s="121"/>
+      <c r="F109" s="121"/>
+      <c r="G109" s="121"/>
+      <c r="H109" s="121"/>
+      <c r="I109" s="121"/>
+      <c r="J109" s="121"/>
+      <c r="K109" s="121"/>
+      <c r="L109" s="121"/>
+    </row>
+    <row r="110" ht="25" customHeight="1">
+      <c r="A110" s="121"/>
+      <c r="B110" s="121"/>
+      <c r="C110" s="121"/>
+      <c r="D110" s="121"/>
+      <c r="E110" s="121"/>
+      <c r="F110" s="121"/>
+      <c r="G110" s="121"/>
+      <c r="H110" s="121"/>
+      <c r="I110" s="121"/>
+      <c r="J110" s="121"/>
+      <c r="K110" s="121"/>
+      <c r="L110" s="121"/>
+    </row>
+    <row r="111" ht="25" customHeight="1">
+      <c r="A111" s="121"/>
+      <c r="B111" s="121"/>
+      <c r="C111" s="121"/>
+      <c r="D111" s="121"/>
+      <c r="E111" s="121"/>
+      <c r="F111" s="121"/>
+      <c r="G111" s="121"/>
+      <c r="H111" s="121"/>
+      <c r="I111" s="121"/>
+      <c r="J111" s="121"/>
+      <c r="K111" s="121"/>
+      <c r="L111" s="121"/>
+    </row>
+    <row r="112" ht="25" customHeight="1">
+      <c r="A112" s="121"/>
+      <c r="B112" s="121"/>
+      <c r="C112" s="121"/>
+      <c r="D112" s="121"/>
+      <c r="E112" s="121"/>
+      <c r="F112" s="121"/>
+      <c r="G112" s="121"/>
+      <c r="H112" s="121"/>
+      <c r="I112" s="121"/>
+      <c r="J112" s="121"/>
+      <c r="K112" s="121"/>
+      <c r="L112" s="121"/>
+    </row>
+    <row r="113" ht="25" customHeight="1">
+      <c r="A113" s="121"/>
+      <c r="B113" s="121"/>
+      <c r="C113" s="121"/>
+      <c r="D113" s="121"/>
+      <c r="E113" s="121"/>
+      <c r="F113" s="121"/>
+      <c r="G113" s="121"/>
+      <c r="H113" s="121"/>
+      <c r="I113" s="121"/>
+      <c r="J113" s="121"/>
+      <c r="K113" s="121"/>
+      <c r="L113" s="121"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="B105:D105"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
+  </hyperlinks>
+  <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.15" footer="0.15"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToWidth="1" fitToHeight="0"/>
+  <tableParts count="1">
+    <tablePart ns1:id="Rbc9541fcab6f4b64"/>
   </tableParts>
 </worksheet>
 </file>
@@ -22426,7 +25511,7 @@
     <mergeCell ref="B100:E100"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -22435,7 +25520,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS2&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R7ccc65d368944179"/>
+    <tablePart ns1:id="R02ce76a9f86743a9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -23644,7 +26729,7 @@
     <mergeCell ref="B28:G28"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -23653,7 +26738,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS3&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="Rb20cb82031ab44c5"/>
+    <tablePart ns1:id="Rff1044c4d2214aa0"/>
   </tableParts>
 </worksheet>
 </file>
@@ -24708,7 +27793,7 @@
     <mergeCell ref="B38:G38"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -24717,7 +27802,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS4&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R8f449789c18c440a"/>
+    <tablePart ns1:id="R9dc9331ec5454a3c"/>
   </tableParts>
 </worksheet>
 </file>
@@ -25313,7 +28398,7 @@
     <mergeCell ref="B24:E24"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -25322,7 +28407,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS5&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R4dbcff9f68df435f"/>
+    <tablePart ns1:id="R371660ae7aae4d55"/>
   </tableParts>
 </worksheet>
 </file>
@@ -28676,7 +31761,7 @@
     <mergeCell ref="B85:G85"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -28685,7 +31770,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS6&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R7b035b02cd9a40a6"/>
+    <tablePart ns1:id="R360651a9cbf74d87"/>
   </tableParts>
 </worksheet>
 </file>
@@ -31357,7 +34442,7 @@
     <mergeCell ref="B57:G57"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -31366,7 +34451,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS7&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R4b434d0cf46840e8"/>
+    <tablePart ns1:id="R92170317539a436e"/>
   </tableParts>
 </worksheet>
 </file>
@@ -38170,7 +41255,7 @@
     <mergeCell ref="B91:G91"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B6" location="'Contents'!B2" display="Contents" tooltip="Return to contents"/>
+    <hyperlink ref="B6" location="'Contents'!B2"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0" horizontalCentered="0"/>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.15" footer="0.2"/>
@@ -38179,7 +41264,7 @@
     <oddFooter>&amp;LPRIDE supplementary tables&amp;CS8&amp;RPage &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <tableParts count="1">
-    <tablePart ns1:id="R39126c0ed6f94ee1"/>
+    <tablePart ns1:id="R015281d9c4794d98"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>